<commit_message>
Record Carl's pre-construction decisions and add a visible contingency line
Folds the ten decisions from 28 Sep 2026 into the proposal (new §9):
fixed DPA fees with a 12-hour addition cap, a customer-visible
contingency, allowances stated as customer prices, designer logging by
phase, a published price guide including kitchens, new terms for the
eight signed PBAs, turnaround ownership, a tier-product grid, the
framing lumber catalog update and "by owner" naming for $0 lines.

§1.3 adds the designer's own logged hours, split into concept work and
construction drawings from the entry notes.

The three ballpark templates now carry one contingency line per tier
(5% / 8% / 10%, a job parameter the estimator sets), mark allowance
lines as price type, and rebuild with the new examples. Calibration
still compares prices before contingency; its results are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ch22kiCEY7KwpDM4Ye9Kr8
</commit_message>
<xml_diff>
--- a/docs/ballpark/kitchen-ballpark-template.xlsx
+++ b/docs/ballpark/kitchen-ballpark-template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId3"/>
@@ -16,14 +16,15 @@
     <sheet name="Calibration" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="LaborCost" vbProcedure="false">Rates!$C$9</definedName>
-    <definedName function="false" hidden="false" name="MarkupCodes" vbProcedure="false">Rates!$A$4:$A$7</definedName>
-    <definedName function="false" hidden="false" name="MarkupVals" vbProcedure="false">Rates!$C$4:$C$7</definedName>
+    <definedName function="false" hidden="false" name="LaborCost" vbProcedure="false">Rates!$C$11</definedName>
+    <definedName function="false" hidden="false" name="MarkupCodes" vbProcedure="false">Rates!$A$4:$A$9</definedName>
+    <definedName function="false" hidden="false" name="MarkupVals" vbProcedure="false">Rates!$C$4:$C$9</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Appliances_Installed" vbProcedure="false">Calculator!$B$11</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Appliances_Supplied" vbProcedure="false">Calculator!$B$10</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Backsplash" vbProcedure="false">Calculator!$B$9</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Cabinet_Run" vbProcedure="false">Calculator!$B$7</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Circuits_Added" vbProcedure="false">Calculator!$B$17</definedName>
+    <definedName function="false" hidden="false" name="p_Kitchen_Contingency_Rate" vbProcedure="false">Calculator!$B$26</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Dumpster_Loads" vbProcedure="false">Calculator!$B$24</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Exterior_Doors" vbProcedure="false">Calculator!$B$22</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Fixtures_Relocated" vbProcedure="false">Calculator!$B$13</definedName>
@@ -40,7 +41,7 @@
     <definedName function="false" hidden="false" name="p_Kitchen_Travel_Hours" vbProcedure="false">Calculator!$B$25</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Under_Cabinet_Lighting" vbProcedure="false">Calculator!$B$18</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Walls_Moved" vbProcedure="false">Calculator!$B$19</definedName>
-    <definedName function="false" hidden="false" name="RangePct" vbProcedure="false">Rates!$C$12</definedName>
+    <definedName function="false" hidden="false" name="RangePct" vbProcedure="false">Rates!$C$14</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -52,12 +53,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="356">
   <si>
     <t xml:space="preserve">Kitchen Ballpark Template — DRAFT for review</t>
   </si>
   <si>
-    <t xml:space="preserve">Deitemeyer Brothers · General Construction · drafted 27 Sep 2026</t>
+    <t xml:space="preserve">Deitemeyer Brothers · General Construction · drafted 27 Sep 2026 · decisions applied 28 Sep 2026</t>
   </si>
   <si>
     <t xml:space="preserve">What this is</t>
@@ -78,7 +79,7 @@
     <t xml:space="preserve">2. Template tab: every JobTread line with its cost group, cost code, unit, exact quantity formula, and unit cost and price per tier.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Parameters tab: the 21 JobTread job parameters. Each starts with 'Kitchen ' so a job with a kitchen and a bath never shares one.</t>
+    <t xml:space="preserve">3. Parameters tab: the 21 site-visit parameters plus the contingency rate, which the estimator sets. Each starts with 'Kitchen ' so a job with a kitchen and a bath never shares one.</t>
   </si>
   <si>
     <t xml:space="preserve">4. Rates tab: markup by cost type, and the ± band. It is set to ±20% for kitchens.</t>
@@ -108,16 +109,19 @@
     <t xml:space="preserve">So the ballpark is quoted at ±20%, as the proposal planned, until three kitchens have closed. Then re-run the calibration and tighten it to ±15%.</t>
   </si>
   <si>
-    <t xml:space="preserve">Decisions still open (for Carl)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allowance type on the selection lines: cost (marked up like other materials, as drafted), price, or cost plus fee.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name the cabinet line, countertop material and backsplash for each tier so sales can show them.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whether DB supplies appliances by default or only on request.</t>
+    <t xml:space="preserve">Decided 28 Sep 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency is its own line on each tier: 8% for a remodel where anything moves, 5% for a refresh that keeps the layout. The estimator sets the Kitchen Contingency Rate. The checks compare prices before contingency, because DB's past estimates carried none.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowances are stated as customer prices (JobTread allowance type: price). No total changes; an overage or a credit is simply the difference in price.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Products per tier: the estimator and the designer name one product per Good / Better / Best cell and lock the grid for six months (draft in the proposal, §9).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still open: whether DB supplies appliances by default or only on request.</t>
   </si>
   <si>
     <t xml:space="preserve">Source for every rate: kitchen estimates read from DB's JobTread account (read-only) on 27 Sep 2026. See Calibration tab.</t>
@@ -222,30 +226,33 @@
     <t xml:space="preserve">{Kitchen Appliances Supplied}</t>
   </si>
   <si>
+    <t xml:space="preserve">Contingency (the Kitchen Contingency Rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kitchen Appliances Installed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All appliances DB sets, including ones the customer buys</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Appliances Installed}</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ballpark total</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Appliances Installed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All appliances DB sets, including ones the customer buys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Appliances Installed}</t>
+    <t xml:space="preserve">Kitchen Fixtures Replaced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plumbing fixtures in the same spot: sink, dishwasher, fridge water line, pot filler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Fixtures Replaced}</t>
   </si>
   <si>
     <t xml:space="preserve">Check: equals Template total</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Fixtures Replaced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plumbing fixtures in the same spot: sink, dishwasher, fridge water line, pot filler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Fixtures Replaced}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kitchen Fixtures Relocated</t>
   </si>
   <si>
@@ -255,42 +262,42 @@
     <t xml:space="preserve">{Kitchen Fixtures Relocated}</t>
   </si>
   <si>
+    <t xml:space="preserve">Kitchen New Flooring Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SF of new flooring, including any beyond the kitchen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen New Flooring Area}</t>
+  </si>
+  <si>
     <t xml:space="preserve">Budget range shown to customer</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen New Flooring Area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SF of new flooring, including any beyond the kitchen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen New Flooring Area}</t>
+    <t xml:space="preserve">Kitchen Light Fixtures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendants or ceiling fixtures replaced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Light Fixtures}</t>
   </si>
   <si>
     <t xml:space="preserve">Low</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Light Fixtures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendants or ceiling fixtures replaced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Light Fixtures}</t>
+    <t xml:space="preserve">Kitchen Recessed Lights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New recessed cans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Recessed Lights}</t>
   </si>
   <si>
     <t xml:space="preserve">High</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Recessed Lights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New recessed cans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Recessed Lights}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kitchen Circuits Added</t>
   </si>
   <si>
@@ -300,30 +307,30 @@
     <t xml:space="preserve">{Kitchen Circuits Added}</t>
   </si>
   <si>
+    <t xml:space="preserve">Kitchen Under-Cabinet Lighting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 = add under-cabinet lighting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Under-Cabinet Lighting}</t>
+  </si>
+  <si>
     <t xml:space="preserve">Totals exclude sales tax and the design agreement fee.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Under-Cabinet Lighting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 = add under-cabinet lighting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Under-Cabinet Lighting}</t>
+    <t xml:space="preserve">Kitchen Walls Moved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walls framed, removed or relocated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Walls Moved}</t>
   </si>
   <si>
     <t xml:space="preserve">The ± band is set on the Rates tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Walls Moved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walls framed, removed or relocated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Walls Moved}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kitchen Subfloor Repair Area</t>
   </si>
   <si>
@@ -378,6 +385,15 @@
     <t xml:space="preserve">{Kitchen Travel Hours}</t>
   </si>
   <si>
+    <t xml:space="preserve">Kitchen Contingency Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency as a % of the tier total, set by the estimator: 5 for a refresh that keeps the layout, 8 when anything moves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Contingency Rate}</t>
+  </si>
+  <si>
     <t xml:space="preserve">JobTread build sheet: cost group "BALLPARK — Kitchen"</t>
   </si>
   <si>
@@ -441,7 +457,7 @@
     <t xml:space="preserve">Best total</t>
   </si>
   <si>
-    <t xml:space="preserve">Allowance line?</t>
+    <t xml:space="preserve">Allowance type</t>
   </si>
   <si>
     <t xml:space="preserve">Note</t>
@@ -744,7 +760,7 @@
     <t xml:space="preserve">Linear Feet</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes</t>
+    <t xml:space="preserve">Price</t>
   </si>
   <si>
     <t xml:space="preserve">Per linear foot of base-cabinet run, uppers and towers included (DB's own convention). Good = stock builder line ($270 price per LF on DB's apartment kitchens). Better = $600 cost, DB's standard cabinet allowance. Best = premium line such as KraftMaid plywood or painted; DB's kitchen addition bid $1,178 price per LF.</t>
@@ -843,6 +859,33 @@
     <t xml:space="preserve">Under-Cabinet Lighting</t>
   </si>
   <si>
+    <t xml:space="preserve">Contingency — Good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Contingency Rate}/100*((1)*275.5 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + ({Kitchen Travel Hours})*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*580 + (4 + ceil(1.1*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*33.35 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*26 + (1)*435 + ({Kitchen Appliances Supplied})*1015 + ({Kitchen New Flooring Area})*5.8 + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000))*100 + ({Kitchen Light Fixtures})*116 + ({Kitchen Recessed Lights})*36.25 + ({Kitchen Under-Cabinet Lighting})*435)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency: the rate times this tier's whole price before contingency. JobTread formulas cannot reference other lines, so the subtotal is spelled out; regenerate this formula (run the build script) after any rate change. Unit price $1.00, cost type Other with markup 0, cost code Contingency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency — Better</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Contingency Rate}/100*((1)*275.5 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + ({Kitchen Travel Hours})*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*870 + (4 + ceil(1.3*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*104 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*45.5 + (1)*870 + ({Kitchen Appliances Supplied})*2030 + ({Kitchen New Flooring Area})*7.25 + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000))*100 + ({Kitchen Light Fixtures})*261 + ({Kitchen Recessed Lights})*50.75 + ({Kitchen Under-Cabinet Lighting})*725)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingency — Best</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Contingency Rate}/100*((1)*275.5 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + ({Kitchen Travel Hours})*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*1305 + (4 + ceil(1.5*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*159.9 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*156 + (1)*1450 + ({Kitchen Appliances Supplied})*3335 + ({Kitchen New Flooring Area})*19.5 + ({Kitchen Light Fixtures})*507.5 + ({Kitchen Recessed Lights})*87 + ({Kitchen Under-Cabinet Lighting})*1116.5)</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
@@ -946,6 +989,18 @@
   </si>
   <si>
     <t xml:space="preserve">Permits and misc. fees: ×1.45.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor, per unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor the catalog prices per square or foot (siding, roofing, gutters). JobTread cost type Labor, marked up ×1.45 like the catalog.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Its own line, carried at cost so it can be reported and credited. JobTread cost type Other with the markup set to 0, cost code Contingency.</t>
   </si>
   <si>
     <t xml:space="preserve">Labor cost per hour</t>
@@ -1629,7 +1684,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -1745,7 +1800,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>19</v>
       </c>
@@ -1761,11 +1816,16 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3"/>
+      <c r="A28" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>22</v>
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1784,7 +1844,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1797,7 +1857,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -1810,7 +1870,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -1834,47 +1894,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>180</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G5" s="14" t="n">
         <f aca="false">SUMIFS(Template!K5:K32,Template!B5:B32,"*Phase 1 -*")</f>
@@ -1891,20 +1951,20 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G6" s="14" t="n">
         <f aca="false">SUMIFS(Template!K5:K32,Template!B5:B32,"*Phase 2 -*")</f>
@@ -1921,20 +1981,20 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>26</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G7" s="14" t="n">
         <f aca="false">SUMIFS(Template!K5:K32,Template!B5:B32,"*Phase 3 -*")</f>
@@ -1951,20 +2011,20 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>6</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" s="14" t="n">
         <f aca="false">SUMIFS(Template!K5:K32,Template!B5:B32,"*Phase 4 -*")</f>
@@ -1981,20 +2041,20 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G9" s="14" t="n">
         <f aca="false">SUM(Template!K33:K46)</f>
@@ -2011,220 +2071,229 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E10" s="6"/>
-      <c r="F10" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10" s="16" t="n">
-        <f aca="false">SUM(G5:G9)</f>
-        <v>41990.96</v>
-      </c>
-      <c r="H10" s="16" t="n">
-        <f aca="false">SUM(H5:H9)</f>
-        <v>56288.61</v>
-      </c>
-      <c r="I10" s="16" t="n">
-        <f aca="false">SUM(I5:I9)</f>
-        <v>77710.51</v>
+      <c r="F10" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <f aca="false">SUM(Template!K47:K49)</f>
+        <v>3359.2768</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <f aca="false">SUM(Template!O47:O49)</f>
+        <v>4503.0888</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <f aca="false">SUM(Template!S47:S49)</f>
+        <v>6216.8408</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>4</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E11" s="6"/>
-      <c r="F11" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G11" s="17" t="str">
-        <f aca="false">IF(ABS(G10-Template!K47)&lt;0.01,"OK","MISMATCH")</f>
-        <v>OK</v>
-      </c>
-      <c r="H11" s="17" t="str">
-        <f aca="false">IF(ABS(H10-Template!O47)&lt;0.01,"OK","MISMATCH")</f>
-        <v>OK</v>
-      </c>
-      <c r="I11" s="17" t="str">
-        <f aca="false">IF(ABS(I10-Template!S47)&lt;0.01,"OK","MISMATCH")</f>
-        <v>OK</v>
+      <c r="F11" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <f aca="false">SUM(G5:G10)</f>
+        <v>45350.2368</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <f aca="false">SUM(H5:H10)</f>
+        <v>60791.6988</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <f aca="false">SUM(I5:I10)</f>
+        <v>83927.3508</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
+      <c r="F12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" s="17" t="str">
+        <f aca="false">IF(ABS(G11-Template!K50)&lt;0.01,"OK","MISMATCH")</f>
+        <v>OK</v>
+      </c>
+      <c r="H12" s="17" t="str">
+        <f aca="false">IF(ABS(H11-Template!O50)&lt;0.01,"OK","MISMATCH")</f>
+        <v>OK</v>
+      </c>
+      <c r="I12" s="17" t="str">
+        <f aca="false">IF(ABS(I11-Template!S50)&lt;0.01,"OK","MISMATCH")</f>
+        <v>OK</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E13" s="6"/>
-      <c r="F13" s="15" t="s">
-        <v>67</v>
-      </c>
+      <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>180</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" s="6"/>
-      <c r="F14" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G14" s="14" t="n">
-        <f aca="false">ROUND(G10*(1-RangePct),-2)</f>
-        <v>33600</v>
-      </c>
-      <c r="H14" s="14" t="n">
-        <f aca="false">ROUND(H10*(1-RangePct),-2)</f>
-        <v>45000</v>
-      </c>
-      <c r="I14" s="14" t="n">
-        <f aca="false">ROUND(I10*(1-RangePct),-2)</f>
-        <v>62200</v>
-      </c>
+      <c r="F14" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G15" s="14" t="n">
-        <f aca="false">ROUND(G10*(1+RangePct),-2)</f>
-        <v>50400</v>
+        <f aca="false">ROUND(G11*(1-RangePct),-2)</f>
+        <v>36300</v>
       </c>
       <c r="H15" s="14" t="n">
-        <f aca="false">ROUND(H10*(1+RangePct),-2)</f>
-        <v>67500</v>
+        <f aca="false">ROUND(H11*(1-RangePct),-2)</f>
+        <v>48600</v>
       </c>
       <c r="I15" s="14" t="n">
-        <f aca="false">ROUND(I10*(1+RangePct),-2)</f>
-        <v>93300</v>
+        <f aca="false">ROUND(I11*(1-RangePct),-2)</f>
+        <v>67100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>6</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
+      <c r="F16" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <f aca="false">ROUND(G11*(1+RangePct),-2)</f>
+        <v>54400</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <f aca="false">ROUND(H11*(1+RangePct),-2)</f>
+        <v>73000</v>
+      </c>
+      <c r="I16" s="14" t="n">
+        <f aca="false">ROUND(I11*(1+RangePct),-2)</f>
+        <v>100700</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E17" s="6"/>
-      <c r="F17" s="7" t="s">
-        <v>82</v>
-      </c>
+      <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
@@ -2232,35 +2301,37 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
+      <c r="F19" s="7" t="s">
+        <v>91</v>
+      </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B20" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -2270,16 +2341,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B21" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -2289,16 +2360,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B22" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
@@ -2308,16 +2379,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B23" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
@@ -2327,16 +2398,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B24" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
@@ -2346,22 +2417,41 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B25" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
       <c r="I25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2379,7 +2469,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U47"/>
+  <dimension ref="A1:U50"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -2395,7 +2485,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2420,7 +2510,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2468,67 +2558,67 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2536,19 +2626,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G5" s="20" t="n">
         <f aca="false">1</f>
@@ -2558,7 +2648,7 @@
         <v>190</v>
       </c>
       <c r="I5" s="22" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="J5" s="23" t="n">
         <f aca="false">H5*INDEX(MarkupVals,MATCH(I5,MarkupCodes,0))</f>
@@ -2572,7 +2662,7 @@
         <v>190</v>
       </c>
       <c r="M5" s="22" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="N5" s="23" t="n">
         <f aca="false">L5*INDEX(MarkupVals,MATCH(M5,MarkupCodes,0))</f>
@@ -2586,7 +2676,7 @@
         <v>190</v>
       </c>
       <c r="Q5" s="22" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="R5" s="23" t="n">
         <f aca="false">P5*INDEX(MarkupVals,MATCH(Q5,MarkupCodes,0))</f>
@@ -2598,7 +2688,7 @@
       </c>
       <c r="T5" s="25"/>
       <c r="U5" s="26" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2606,19 +2696,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G6" s="20" t="n">
         <f aca="false">4 + 4*p_Kitchen_Full_Gut</f>
@@ -2629,7 +2719,7 @@
         <v>55</v>
       </c>
       <c r="I6" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">H6*INDEX(MarkupVals,MATCH(I6,MarkupCodes,0))</f>
@@ -2644,7 +2734,7 @@
         <v>55</v>
       </c>
       <c r="M6" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N6" s="23" t="n">
         <f aca="false">L6*INDEX(MarkupVals,MATCH(M6,MarkupCodes,0))</f>
@@ -2659,7 +2749,7 @@
         <v>55</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R6" s="23" t="n">
         <f aca="false">P6*INDEX(MarkupVals,MATCH(Q6,MarkupCodes,0))</f>
@@ -2677,19 +2767,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">1</f>
@@ -2699,7 +2789,7 @@
         <v>150</v>
       </c>
       <c r="I7" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J7" s="23" t="n">
         <f aca="false">H7*INDEX(MarkupVals,MATCH(I7,MarkupCodes,0))</f>
@@ -2713,7 +2803,7 @@
         <v>150</v>
       </c>
       <c r="M7" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N7" s="23" t="n">
         <f aca="false">L7*INDEX(MarkupVals,MATCH(M7,MarkupCodes,0))</f>
@@ -2727,7 +2817,7 @@
         <v>150</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R7" s="23" t="n">
         <f aca="false">P7*INDEX(MarkupVals,MATCH(Q7,MarkupCodes,0))</f>
@@ -2745,19 +2835,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G8" s="20" t="n">
         <f aca="false">2</f>
@@ -2768,7 +2858,7 @@
         <v>55</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J8" s="23" t="n">
         <f aca="false">H8*INDEX(MarkupVals,MATCH(I8,MarkupCodes,0))</f>
@@ -2783,7 +2873,7 @@
         <v>55</v>
       </c>
       <c r="M8" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N8" s="23" t="n">
         <f aca="false">L8*INDEX(MarkupVals,MATCH(M8,MarkupCodes,0))</f>
@@ -2798,7 +2888,7 @@
         <v>55</v>
       </c>
       <c r="Q8" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R8" s="23" t="n">
         <f aca="false">P8*INDEX(MarkupVals,MATCH(Q8,MarkupCodes,0))</f>
@@ -2816,19 +2906,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G9" s="20" t="n">
         <f aca="false">8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved</f>
@@ -2839,7 +2929,7 @@
         <v>55</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J9" s="23" t="n">
         <f aca="false">H9*INDEX(MarkupVals,MATCH(I9,MarkupCodes,0))</f>
@@ -2854,7 +2944,7 @@
         <v>55</v>
       </c>
       <c r="M9" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N9" s="23" t="n">
         <f aca="false">L9*INDEX(MarkupVals,MATCH(M9,MarkupCodes,0))</f>
@@ -2869,7 +2959,7 @@
         <v>55</v>
       </c>
       <c r="Q9" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R9" s="23" t="n">
         <f aca="false">P9*INDEX(MarkupVals,MATCH(Q9,MarkupCodes,0))</f>
@@ -2881,7 +2971,7 @@
       </c>
       <c r="T9" s="25"/>
       <c r="U9" s="26" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2889,19 +2979,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G10" s="20" t="n">
         <f aca="false">p_Kitchen_Dumpster_Loads</f>
@@ -2911,7 +3001,7 @@
         <v>250</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J10" s="21" t="n">
         <v>450</v>
@@ -2924,7 +3014,7 @@
         <v>250</v>
       </c>
       <c r="M10" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N10" s="21" t="n">
         <v>450</v>
@@ -2937,7 +3027,7 @@
         <v>250</v>
       </c>
       <c r="Q10" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R10" s="21" t="n">
         <v>450</v>
@@ -2948,7 +3038,7 @@
       </c>
       <c r="T10" s="25"/>
       <c r="U10" s="26" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2956,19 +3046,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="G11" s="20" t="n">
         <f aca="false">2 + 2*p_Kitchen_Full_Gut</f>
@@ -2979,7 +3069,7 @@
         <v>55</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">H11*INDEX(MarkupVals,MATCH(I11,MarkupCodes,0))</f>
@@ -2994,7 +3084,7 @@
         <v>55</v>
       </c>
       <c r="M11" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N11" s="23" t="n">
         <f aca="false">L11*INDEX(MarkupVals,MATCH(M11,MarkupCodes,0))</f>
@@ -3009,7 +3099,7 @@
         <v>55</v>
       </c>
       <c r="Q11" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R11" s="23" t="n">
         <f aca="false">P11*INDEX(MarkupVals,MATCH(Q11,MarkupCodes,0))</f>
@@ -3027,19 +3117,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G12" s="20" t="n">
         <f aca="false">p_Kitchen_Travel_Hours</f>
@@ -3050,7 +3140,7 @@
         <v>55</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">H12*INDEX(MarkupVals,MATCH(I12,MarkupCodes,0))</f>
@@ -3065,7 +3155,7 @@
         <v>55</v>
       </c>
       <c r="M12" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N12" s="23" t="n">
         <f aca="false">L12*INDEX(MarkupVals,MATCH(M12,MarkupCodes,0))</f>
@@ -3080,7 +3170,7 @@
         <v>55</v>
       </c>
       <c r="Q12" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R12" s="23" t="n">
         <f aca="false">P12*INDEX(MarkupVals,MATCH(Q12,MarkupCodes,0))</f>
@@ -3098,19 +3188,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="G13" s="20" t="n">
         <f aca="false">p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0)</f>
@@ -3120,7 +3210,7 @@
         <v>150</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J13" s="23" t="n">
         <f aca="false">H13*INDEX(MarkupVals,MATCH(I13,MarkupCodes,0))</f>
@@ -3134,7 +3224,7 @@
         <v>150</v>
       </c>
       <c r="M13" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N13" s="23" t="n">
         <f aca="false">L13*INDEX(MarkupVals,MATCH(M13,MarkupCodes,0))</f>
@@ -3148,7 +3238,7 @@
         <v>150</v>
       </c>
       <c r="Q13" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R13" s="23" t="n">
         <f aca="false">P13*INDEX(MarkupVals,MATCH(Q13,MarkupCodes,0))</f>
@@ -3166,19 +3256,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="G14" s="20" t="n">
         <f aca="false">4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0)</f>
@@ -3189,7 +3279,7 @@
         <v>55</v>
       </c>
       <c r="I14" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J14" s="23" t="n">
         <f aca="false">H14*INDEX(MarkupVals,MATCH(I14,MarkupCodes,0))</f>
@@ -3204,7 +3294,7 @@
         <v>55</v>
       </c>
       <c r="M14" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N14" s="23" t="n">
         <f aca="false">L14*INDEX(MarkupVals,MATCH(M14,MarkupCodes,0))</f>
@@ -3219,7 +3309,7 @@
         <v>55</v>
       </c>
       <c r="Q14" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R14" s="23" t="n">
         <f aca="false">P14*INDEX(MarkupVals,MATCH(Q14,MarkupCodes,0))</f>
@@ -3237,19 +3327,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G15" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated</f>
@@ -3259,7 +3349,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J15" s="23" t="n">
         <f aca="false">H15*INDEX(MarkupVals,MATCH(I15,MarkupCodes,0))</f>
@@ -3273,7 +3363,7 @@
         <v>100</v>
       </c>
       <c r="M15" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N15" s="23" t="n">
         <f aca="false">L15*INDEX(MarkupVals,MATCH(M15,MarkupCodes,0))</f>
@@ -3287,7 +3377,7 @@
         <v>100</v>
       </c>
       <c r="Q15" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R15" s="23" t="n">
         <f aca="false">P15*INDEX(MarkupVals,MATCH(Q15,MarkupCodes,0))</f>
@@ -3299,7 +3389,7 @@
       </c>
       <c r="T15" s="25"/>
       <c r="U15" s="26" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3307,19 +3397,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="G16" s="20" t="n">
         <f aca="false">3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated</f>
@@ -3330,7 +3420,7 @@
         <v>55</v>
       </c>
       <c r="I16" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J16" s="23" t="n">
         <f aca="false">H16*INDEX(MarkupVals,MATCH(I16,MarkupCodes,0))</f>
@@ -3345,7 +3435,7 @@
         <v>55</v>
       </c>
       <c r="M16" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N16" s="23" t="n">
         <f aca="false">L16*INDEX(MarkupVals,MATCH(M16,MarkupCodes,0))</f>
@@ -3360,7 +3450,7 @@
         <v>55</v>
       </c>
       <c r="Q16" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R16" s="23" t="n">
         <f aca="false">P16*INDEX(MarkupVals,MATCH(Q16,MarkupCodes,0))</f>
@@ -3378,19 +3468,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C17" s="18" t="s">
+        <v>184</v>
+      </c>
+      <c r="D17" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>174</v>
-      </c>
       <c r="E17" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G17" s="20" t="n">
         <f aca="false">p_Kitchen_HVAC_Work</f>
@@ -3400,7 +3490,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J17" s="23" t="n">
         <f aca="false">H17*INDEX(MarkupVals,MATCH(I17,MarkupCodes,0))</f>
@@ -3414,7 +3504,7 @@
         <v>100</v>
       </c>
       <c r="M17" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N17" s="23" t="n">
         <f aca="false">L17*INDEX(MarkupVals,MATCH(M17,MarkupCodes,0))</f>
@@ -3428,7 +3518,7 @@
         <v>100</v>
       </c>
       <c r="Q17" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R17" s="23" t="n">
         <f aca="false">P17*INDEX(MarkupVals,MATCH(Q17,MarkupCodes,0))</f>
@@ -3446,19 +3536,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="G18" s="20" t="n">
         <f aca="false">2*p_Kitchen_HVAC_Work</f>
@@ -3469,7 +3559,7 @@
         <v>55</v>
       </c>
       <c r="I18" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J18" s="23" t="n">
         <f aca="false">H18*INDEX(MarkupVals,MATCH(I18,MarkupCodes,0))</f>
@@ -3484,7 +3574,7 @@
         <v>55</v>
       </c>
       <c r="M18" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N18" s="23" t="n">
         <f aca="false">L18*INDEX(MarkupVals,MATCH(M18,MarkupCodes,0))</f>
@@ -3499,7 +3589,7 @@
         <v>55</v>
       </c>
       <c r="Q18" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R18" s="23" t="n">
         <f aca="false">P18*INDEX(MarkupVals,MATCH(Q18,MarkupCodes,0))</f>
@@ -3517,19 +3607,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G19" s="20" t="n">
         <f aca="false">p_Kitchen_Floor_Area</f>
@@ -3539,7 +3629,7 @@
         <v>2.61</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J19" s="23" t="n">
         <f aca="false">H19*INDEX(MarkupVals,MATCH(I19,MarkupCodes,0))</f>
@@ -3553,7 +3643,7 @@
         <v>2.61</v>
       </c>
       <c r="M19" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N19" s="23" t="n">
         <f aca="false">L19*INDEX(MarkupVals,MATCH(M19,MarkupCodes,0))</f>
@@ -3567,7 +3657,7 @@
         <v>2.61</v>
       </c>
       <c r="Q19" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R19" s="23" t="n">
         <f aca="false">P19*INDEX(MarkupVals,MATCH(Q19,MarkupCodes,0))</f>
@@ -3579,7 +3669,7 @@
       </c>
       <c r="T19" s="25"/>
       <c r="U19" s="26" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,19 +3677,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="G20" s="20" t="n">
         <f aca="false">4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting</f>
@@ -3610,7 +3700,7 @@
         <v>55</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J20" s="23" t="n">
         <f aca="false">H20*INDEX(MarkupVals,MATCH(I20,MarkupCodes,0))</f>
@@ -3625,7 +3715,7 @@
         <v>55</v>
       </c>
       <c r="M20" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N20" s="23" t="n">
         <f aca="false">L20*INDEX(MarkupVals,MATCH(M20,MarkupCodes,0))</f>
@@ -3640,7 +3730,7 @@
         <v>55</v>
       </c>
       <c r="Q20" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R20" s="23" t="n">
         <f aca="false">P20*INDEX(MarkupVals,MATCH(Q20,MarkupCodes,0))</f>
@@ -3658,19 +3748,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="G21" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0)</f>
@@ -3680,7 +3770,7 @@
         <v>23</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J21" s="23" t="n">
         <f aca="false">H21*INDEX(MarkupVals,MATCH(I21,MarkupCodes,0))</f>
@@ -3694,7 +3784,7 @@
         <v>23</v>
       </c>
       <c r="M21" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N21" s="23" t="n">
         <f aca="false">L21*INDEX(MarkupVals,MATCH(M21,MarkupCodes,0))</f>
@@ -3708,7 +3798,7 @@
         <v>23</v>
       </c>
       <c r="Q21" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R21" s="23" t="n">
         <f aca="false">P21*INDEX(MarkupVals,MATCH(Q21,MarkupCodes,0))</f>
@@ -3720,7 +3810,7 @@
       </c>
       <c r="T21" s="25"/>
       <c r="U21" s="26" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3728,19 +3818,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="G22" s="20" t="n">
         <f aca="false">6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0)</f>
@@ -3751,7 +3841,7 @@
         <v>55</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J22" s="23" t="n">
         <f aca="false">H22*INDEX(MarkupVals,MATCH(I22,MarkupCodes,0))</f>
@@ -3766,7 +3856,7 @@
         <v>55</v>
       </c>
       <c r="M22" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N22" s="23" t="n">
         <f aca="false">L22*INDEX(MarkupVals,MATCH(M22,MarkupCodes,0))</f>
@@ -3781,7 +3871,7 @@
         <v>55</v>
       </c>
       <c r="Q22" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R22" s="23" t="n">
         <f aca="false">P22*INDEX(MarkupVals,MATCH(Q22,MarkupCodes,0))</f>
@@ -3799,19 +3889,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Full_Gut</f>
@@ -3821,7 +3911,7 @@
         <v>115</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J23" s="23" t="n">
         <f aca="false">H23*INDEX(MarkupVals,MATCH(I23,MarkupCodes,0))</f>
@@ -3835,7 +3925,7 @@
         <v>115</v>
       </c>
       <c r="M23" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N23" s="23" t="n">
         <f aca="false">L23*INDEX(MarkupVals,MATCH(M23,MarkupCodes,0))</f>
@@ -3849,7 +3939,7 @@
         <v>115</v>
       </c>
       <c r="Q23" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R23" s="23" t="n">
         <f aca="false">P23*INDEX(MarkupVals,MATCH(Q23,MarkupCodes,0))</f>
@@ -3867,19 +3957,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G24" s="20" t="n">
         <f aca="false">3 + ROUNDUP(p_Kitchen_Floor_Area/20,0)</f>
@@ -3890,7 +3980,7 @@
         <v>55</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J24" s="23" t="n">
         <f aca="false">H24*INDEX(MarkupVals,MATCH(I24,MarkupCodes,0))</f>
@@ -3905,7 +3995,7 @@
         <v>55</v>
       </c>
       <c r="M24" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N24" s="23" t="n">
         <f aca="false">L24*INDEX(MarkupVals,MATCH(M24,MarkupCodes,0))</f>
@@ -3920,7 +4010,7 @@
         <v>55</v>
       </c>
       <c r="Q24" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R24" s="23" t="n">
         <f aca="false">P24*INDEX(MarkupVals,MATCH(Q24,MarkupCodes,0))</f>
@@ -3938,19 +4028,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G25" s="20" t="n">
         <f aca="false">p_Kitchen_New_Flooring_Area</f>
@@ -3960,7 +4050,7 @@
         <v>0.75</v>
       </c>
       <c r="I25" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J25" s="23" t="n">
         <f aca="false">H25*INDEX(MarkupVals,MATCH(I25,MarkupCodes,0))</f>
@@ -3974,7 +4064,7 @@
         <v>0.75</v>
       </c>
       <c r="M25" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N25" s="23" t="n">
         <f aca="false">L25*INDEX(MarkupVals,MATCH(M25,MarkupCodes,0))</f>
@@ -3988,7 +4078,7 @@
         <v>0.75</v>
       </c>
       <c r="Q25" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R25" s="23" t="n">
         <f aca="false">P25*INDEX(MarkupVals,MATCH(Q25,MarkupCodes,0))</f>
@@ -4006,19 +4096,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="G26" s="20" t="n">
         <f aca="false">ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0)</f>
@@ -4028,7 +4118,7 @@
         <v>10</v>
       </c>
       <c r="I26" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J26" s="23" t="n">
         <f aca="false">H26*INDEX(MarkupVals,MATCH(I26,MarkupCodes,0))</f>
@@ -4042,7 +4132,7 @@
         <v>10</v>
       </c>
       <c r="M26" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N26" s="23" t="n">
         <f aca="false">L26*INDEX(MarkupVals,MATCH(M26,MarkupCodes,0))</f>
@@ -4056,7 +4146,7 @@
         <v>10</v>
       </c>
       <c r="Q26" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R26" s="23" t="n">
         <f aca="false">P26*INDEX(MarkupVals,MATCH(Q26,MarkupCodes,0))</f>
@@ -4074,19 +4164,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="G27" s="20" t="n">
         <f aca="false">2*p_Kitchen_Appliances_Installed</f>
@@ -4097,7 +4187,7 @@
         <v>55</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J27" s="23" t="n">
         <f aca="false">H27*INDEX(MarkupVals,MATCH(I27,MarkupCodes,0))</f>
@@ -4112,7 +4202,7 @@
         <v>55</v>
       </c>
       <c r="M27" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N27" s="23" t="n">
         <f aca="false">L27*INDEX(MarkupVals,MATCH(M27,MarkupCodes,0))</f>
@@ -4127,7 +4217,7 @@
         <v>55</v>
       </c>
       <c r="Q27" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R27" s="23" t="n">
         <f aca="false">P27*INDEX(MarkupVals,MATCH(Q27,MarkupCodes,0))</f>
@@ -4139,7 +4229,7 @@
       </c>
       <c r="T27" s="25"/>
       <c r="U27" s="26" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4147,19 +4237,19 @@
         <v>24</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G28" s="20" t="n">
         <f aca="false">p_Kitchen_Interior_Doors</f>
@@ -4169,7 +4259,7 @@
         <v>400</v>
       </c>
       <c r="I28" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J28" s="23" t="n">
         <f aca="false">H28*INDEX(MarkupVals,MATCH(I28,MarkupCodes,0))</f>
@@ -4183,7 +4273,7 @@
         <v>400</v>
       </c>
       <c r="M28" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N28" s="23" t="n">
         <f aca="false">L28*INDEX(MarkupVals,MATCH(M28,MarkupCodes,0))</f>
@@ -4197,7 +4287,7 @@
         <v>400</v>
       </c>
       <c r="Q28" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R28" s="23" t="n">
         <f aca="false">P28*INDEX(MarkupVals,MATCH(Q28,MarkupCodes,0))</f>
@@ -4215,19 +4305,19 @@
         <v>25</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G29" s="20" t="n">
         <f aca="false">p_Kitchen_Exterior_Doors</f>
@@ -4237,7 +4327,7 @@
         <v>1230</v>
       </c>
       <c r="I29" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J29" s="23" t="n">
         <f aca="false">H29*INDEX(MarkupVals,MATCH(I29,MarkupCodes,0))</f>
@@ -4251,7 +4341,7 @@
         <v>1230</v>
       </c>
       <c r="M29" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N29" s="23" t="n">
         <f aca="false">L29*INDEX(MarkupVals,MATCH(M29,MarkupCodes,0))</f>
@@ -4265,7 +4355,7 @@
         <v>1230</v>
       </c>
       <c r="Q29" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R29" s="23" t="n">
         <f aca="false">P29*INDEX(MarkupVals,MATCH(Q29,MarkupCodes,0))</f>
@@ -4277,7 +4367,7 @@
       </c>
       <c r="T29" s="25"/>
       <c r="U29" s="26" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4285,19 +4375,19 @@
         <v>26</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="G30" s="20" t="n">
         <f aca="false">3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors</f>
@@ -4308,7 +4398,7 @@
         <v>55</v>
       </c>
       <c r="I30" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J30" s="23" t="n">
         <f aca="false">H30*INDEX(MarkupVals,MATCH(I30,MarkupCodes,0))</f>
@@ -4323,7 +4413,7 @@
         <v>55</v>
       </c>
       <c r="M30" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N30" s="23" t="n">
         <f aca="false">L30*INDEX(MarkupVals,MATCH(M30,MarkupCodes,0))</f>
@@ -4338,7 +4428,7 @@
         <v>55</v>
       </c>
       <c r="Q30" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R30" s="23" t="n">
         <f aca="false">P30*INDEX(MarkupVals,MATCH(Q30,MarkupCodes,0))</f>
@@ -4356,19 +4446,19 @@
         <v>27</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="G31" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0)</f>
@@ -4378,7 +4468,7 @@
         <v>20</v>
       </c>
       <c r="I31" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J31" s="23" t="n">
         <f aca="false">H31*INDEX(MarkupVals,MATCH(I31,MarkupCodes,0))</f>
@@ -4392,7 +4482,7 @@
         <v>20</v>
       </c>
       <c r="M31" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N31" s="23" t="n">
         <f aca="false">L31*INDEX(MarkupVals,MATCH(M31,MarkupCodes,0))</f>
@@ -4406,7 +4496,7 @@
         <v>20</v>
       </c>
       <c r="Q31" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R31" s="23" t="n">
         <f aca="false">P31*INDEX(MarkupVals,MATCH(Q31,MarkupCodes,0))</f>
@@ -4424,19 +4514,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="G32" s="20" t="n">
         <f aca="false">2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors</f>
@@ -4447,7 +4537,7 @@
         <v>55</v>
       </c>
       <c r="I32" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J32" s="23" t="n">
         <f aca="false">H32*INDEX(MarkupVals,MATCH(I32,MarkupCodes,0))</f>
@@ -4462,7 +4552,7 @@
         <v>55</v>
       </c>
       <c r="M32" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N32" s="23" t="n">
         <f aca="false">L32*INDEX(MarkupVals,MATCH(M32,MarkupCodes,0))</f>
@@ -4477,7 +4567,7 @@
         <v>55</v>
       </c>
       <c r="Q32" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R32" s="23" t="n">
         <f aca="false">P32*INDEX(MarkupVals,MATCH(Q32,MarkupCodes,0))</f>
@@ -4495,19 +4585,19 @@
         <v>29</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G33" s="20" t="n">
         <f aca="false">p_Kitchen_Cabinet_Run</f>
@@ -4517,7 +4607,7 @@
         <v>400</v>
       </c>
       <c r="I33" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J33" s="23" t="n">
         <f aca="false">H33*INDEX(MarkupVals,MATCH(I33,MarkupCodes,0))</f>
@@ -4531,7 +4621,7 @@
         <v>600</v>
       </c>
       <c r="M33" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N33" s="23" t="n">
         <f aca="false">L33*INDEX(MarkupVals,MATCH(M33,MarkupCodes,0))</f>
@@ -4545,7 +4635,7 @@
         <v>900</v>
       </c>
       <c r="Q33" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R33" s="23" t="n">
         <f aca="false">P33*INDEX(MarkupVals,MATCH(Q33,MarkupCodes,0))</f>
@@ -4556,10 +4646,10 @@
         <v>33930</v>
       </c>
       <c r="T33" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U33" s="26" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4567,19 +4657,19 @@
         <v>30</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="G34" s="20" t="n">
         <f aca="false">4 + ROUNDUP(1.1*p_Kitchen_Cabinet_Run,0)</f>
@@ -4590,7 +4680,7 @@
         <v>55</v>
       </c>
       <c r="I34" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J34" s="23" t="n">
         <f aca="false">H34*INDEX(MarkupVals,MATCH(I34,MarkupCodes,0))</f>
@@ -4604,7 +4694,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N34" s="23" t="n">
         <f aca="false">L34*INDEX(MarkupVals,MATCH(M34,MarkupCodes,0))</f>
@@ -4618,7 +4708,7 @@
         <v>0</v>
       </c>
       <c r="Q34" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R34" s="23" t="n">
         <f aca="false">P34*INDEX(MarkupVals,MATCH(Q34,MarkupCodes,0))</f>
@@ -4630,7 +4720,7 @@
       </c>
       <c r="T34" s="25"/>
       <c r="U34" s="26" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4638,19 +4728,19 @@
         <v>31</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="G35" s="20" t="n">
         <f aca="false">4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0)</f>
@@ -4660,7 +4750,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J35" s="23" t="n">
         <f aca="false">H35*INDEX(MarkupVals,MATCH(I35,MarkupCodes,0))</f>
@@ -4675,7 +4765,7 @@
         <v>55</v>
       </c>
       <c r="M35" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N35" s="23" t="n">
         <f aca="false">L35*INDEX(MarkupVals,MATCH(M35,MarkupCodes,0))</f>
@@ -4689,7 +4779,7 @@
         <v>0</v>
       </c>
       <c r="Q35" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R35" s="23" t="n">
         <f aca="false">P35*INDEX(MarkupVals,MATCH(Q35,MarkupCodes,0))</f>
@@ -4701,7 +4791,7 @@
       </c>
       <c r="T35" s="25"/>
       <c r="U35" s="26" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4709,19 +4799,19 @@
         <v>32</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="G36" s="20" t="n">
         <f aca="false">4 + ROUNDUP(1.5*p_Kitchen_Cabinet_Run,0)</f>
@@ -4731,7 +4821,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J36" s="23" t="n">
         <f aca="false">H36*INDEX(MarkupVals,MATCH(I36,MarkupCodes,0))</f>
@@ -4745,7 +4835,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N36" s="23" t="n">
         <f aca="false">L36*INDEX(MarkupVals,MATCH(M36,MarkupCodes,0))</f>
@@ -4760,7 +4850,7 @@
         <v>55</v>
       </c>
       <c r="Q36" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R36" s="23" t="n">
         <f aca="false">P36*INDEX(MarkupVals,MATCH(Q36,MarkupCodes,0))</f>
@@ -4772,7 +4862,7 @@
       </c>
       <c r="T36" s="25"/>
       <c r="U36" s="26" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4780,19 +4870,19 @@
         <v>33</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="G37" s="20" t="n">
         <f aca="false">2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0)</f>
@@ -4802,7 +4892,7 @@
         <v>23</v>
       </c>
       <c r="I37" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J37" s="23" t="n">
         <f aca="false">H37*INDEX(MarkupVals,MATCH(I37,MarkupCodes,0))</f>
@@ -4816,7 +4906,7 @@
         <v>80</v>
       </c>
       <c r="M37" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="N37" s="23" t="n">
         <f aca="false">L37*INDEX(MarkupVals,MATCH(M37,MarkupCodes,0))</f>
@@ -4830,7 +4920,7 @@
         <v>123</v>
       </c>
       <c r="Q37" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="R37" s="23" t="n">
         <f aca="false">P37*INDEX(MarkupVals,MATCH(Q37,MarkupCodes,0))</f>
@@ -4841,10 +4931,10 @@
         <v>9753.9</v>
       </c>
       <c r="T37" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U37" s="26" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4852,19 +4942,19 @@
         <v>34</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G38" s="20" t="n">
         <f aca="false">p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0)</f>
@@ -4874,7 +4964,7 @@
         <v>20</v>
       </c>
       <c r="I38" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="J38" s="23" t="n">
         <f aca="false">H38*INDEX(MarkupVals,MATCH(I38,MarkupCodes,0))</f>
@@ -4888,7 +4978,7 @@
         <v>35</v>
       </c>
       <c r="M38" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="N38" s="23" t="n">
         <f aca="false">L38*INDEX(MarkupVals,MATCH(M38,MarkupCodes,0))</f>
@@ -4902,7 +4992,7 @@
         <v>120</v>
       </c>
       <c r="Q38" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="R38" s="23" t="n">
         <f aca="false">P38*INDEX(MarkupVals,MATCH(Q38,MarkupCodes,0))</f>
@@ -4913,10 +5003,10 @@
         <v>4680</v>
       </c>
       <c r="T38" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U38" s="26" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4924,19 +5014,19 @@
         <v>35</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="G39" s="20" t="n">
         <f aca="false">1</f>
@@ -4946,7 +5036,7 @@
         <v>300</v>
       </c>
       <c r="I39" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J39" s="23" t="n">
         <f aca="false">H39*INDEX(MarkupVals,MATCH(I39,MarkupCodes,0))</f>
@@ -4960,7 +5050,7 @@
         <v>600</v>
       </c>
       <c r="M39" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N39" s="23" t="n">
         <f aca="false">L39*INDEX(MarkupVals,MATCH(M39,MarkupCodes,0))</f>
@@ -4974,7 +5064,7 @@
         <v>1000</v>
       </c>
       <c r="Q39" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R39" s="23" t="n">
         <f aca="false">P39*INDEX(MarkupVals,MATCH(Q39,MarkupCodes,0))</f>
@@ -4985,7 +5075,7 @@
         <v>1450</v>
       </c>
       <c r="T39" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U39" s="26"/>
     </row>
@@ -4994,19 +5084,19 @@
         <v>36</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G40" s="20" t="n">
         <f aca="false">p_Kitchen_Appliances_Supplied</f>
@@ -5016,7 +5106,7 @@
         <v>700</v>
       </c>
       <c r="I40" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J40" s="23" t="n">
         <f aca="false">H40*INDEX(MarkupVals,MATCH(I40,MarkupCodes,0))</f>
@@ -5030,7 +5120,7 @@
         <v>1400</v>
       </c>
       <c r="M40" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N40" s="23" t="n">
         <f aca="false">L40*INDEX(MarkupVals,MATCH(M40,MarkupCodes,0))</f>
@@ -5044,7 +5134,7 @@
         <v>2300</v>
       </c>
       <c r="Q40" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R40" s="23" t="n">
         <f aca="false">P40*INDEX(MarkupVals,MATCH(Q40,MarkupCodes,0))</f>
@@ -5055,10 +5145,10 @@
         <v>0</v>
       </c>
       <c r="T40" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U40" s="26" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5066,19 +5156,19 @@
         <v>37</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C41" s="18" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G41" s="20" t="n">
         <f aca="false">p_Kitchen_New_Flooring_Area</f>
@@ -5088,7 +5178,7 @@
         <v>4</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J41" s="23" t="n">
         <f aca="false">H41*INDEX(MarkupVals,MATCH(I41,MarkupCodes,0))</f>
@@ -5102,7 +5192,7 @@
         <v>5</v>
       </c>
       <c r="M41" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N41" s="23" t="n">
         <f aca="false">L41*INDEX(MarkupVals,MATCH(M41,MarkupCodes,0))</f>
@@ -5116,7 +5206,7 @@
         <v>15</v>
       </c>
       <c r="Q41" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="R41" s="23" t="n">
         <f aca="false">P41*INDEX(MarkupVals,MATCH(Q41,MarkupCodes,0))</f>
@@ -5127,10 +5217,10 @@
         <v>3510</v>
       </c>
       <c r="T41" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U41" s="26" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5138,19 +5228,19 @@
         <v>38</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D42" s="18" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G42" s="20" t="n">
         <f aca="false">ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)</f>
@@ -5161,7 +5251,7 @@
         <v>55</v>
       </c>
       <c r="I42" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J42" s="23" t="n">
         <f aca="false">H42*INDEX(MarkupVals,MATCH(I42,MarkupCodes,0))</f>
@@ -5175,7 +5265,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N42" s="23" t="n">
         <f aca="false">L42*INDEX(MarkupVals,MATCH(M42,MarkupCodes,0))</f>
@@ -5189,7 +5279,7 @@
         <v>0</v>
       </c>
       <c r="Q42" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R42" s="23" t="n">
         <f aca="false">P42*INDEX(MarkupVals,MATCH(Q42,MarkupCodes,0))</f>
@@ -5201,7 +5291,7 @@
       </c>
       <c r="T42" s="25"/>
       <c r="U42" s="26" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5209,19 +5299,19 @@
         <v>39</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C43" s="18" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D43" s="18" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="E43" s="18" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G43" s="20" t="n">
         <f aca="false">ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)</f>
@@ -5231,7 +5321,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J43" s="23" t="n">
         <f aca="false">H43*INDEX(MarkupVals,MATCH(I43,MarkupCodes,0))</f>
@@ -5246,7 +5336,7 @@
         <v>55</v>
       </c>
       <c r="M43" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="N43" s="23" t="n">
         <f aca="false">L43*INDEX(MarkupVals,MATCH(M43,MarkupCodes,0))</f>
@@ -5260,7 +5350,7 @@
         <v>0</v>
       </c>
       <c r="Q43" s="22" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="R43" s="23" t="n">
         <f aca="false">P43*INDEX(MarkupVals,MATCH(Q43,MarkupCodes,0))</f>
@@ -5272,7 +5362,7 @@
       </c>
       <c r="T43" s="25"/>
       <c r="U43" s="26" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5280,19 +5370,19 @@
         <v>40</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D44" s="18" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G44" s="20" t="n">
         <f aca="false">p_Kitchen_Light_Fixtures</f>
@@ -5302,7 +5392,7 @@
         <v>80</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J44" s="23" t="n">
         <f aca="false">H44*INDEX(MarkupVals,MATCH(I44,MarkupCodes,0))</f>
@@ -5316,7 +5406,7 @@
         <v>180</v>
       </c>
       <c r="M44" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N44" s="23" t="n">
         <f aca="false">L44*INDEX(MarkupVals,MATCH(M44,MarkupCodes,0))</f>
@@ -5330,7 +5420,7 @@
         <v>350</v>
       </c>
       <c r="Q44" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R44" s="23" t="n">
         <f aca="false">P44*INDEX(MarkupVals,MATCH(Q44,MarkupCodes,0))</f>
@@ -5341,7 +5431,7 @@
         <v>1015</v>
       </c>
       <c r="T44" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U44" s="26"/>
     </row>
@@ -5350,19 +5440,19 @@
         <v>41</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E45" s="18" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G45" s="20" t="n">
         <f aca="false">p_Kitchen_Recessed_Lights</f>
@@ -5372,7 +5462,7 @@
         <v>25</v>
       </c>
       <c r="I45" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J45" s="23" t="n">
         <f aca="false">H45*INDEX(MarkupVals,MATCH(I45,MarkupCodes,0))</f>
@@ -5386,7 +5476,7 @@
         <v>35</v>
       </c>
       <c r="M45" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N45" s="23" t="n">
         <f aca="false">L45*INDEX(MarkupVals,MATCH(M45,MarkupCodes,0))</f>
@@ -5400,7 +5490,7 @@
         <v>60</v>
       </c>
       <c r="Q45" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R45" s="23" t="n">
         <f aca="false">P45*INDEX(MarkupVals,MATCH(Q45,MarkupCodes,0))</f>
@@ -5411,7 +5501,7 @@
         <v>522</v>
       </c>
       <c r="T45" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U45" s="26"/>
     </row>
@@ -5420,19 +5510,19 @@
         <v>42</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E46" s="18" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G46" s="20" t="n">
         <f aca="false">p_Kitchen_Under_Cabinet_Lighting</f>
@@ -5442,7 +5532,7 @@
         <v>300</v>
       </c>
       <c r="I46" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="J46" s="23" t="n">
         <f aca="false">H46*INDEX(MarkupVals,MATCH(I46,MarkupCodes,0))</f>
@@ -5456,7 +5546,7 @@
         <v>500</v>
       </c>
       <c r="M46" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="N46" s="23" t="n">
         <f aca="false">L46*INDEX(MarkupVals,MATCH(M46,MarkupCodes,0))</f>
@@ -5470,7 +5560,7 @@
         <v>770</v>
       </c>
       <c r="Q46" s="22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="R46" s="23" t="n">
         <f aca="false">P46*INDEX(MarkupVals,MATCH(Q46,MarkupCodes,0))</f>
@@ -5481,43 +5571,253 @@
         <v>1116.5</v>
       </c>
       <c r="T46" s="25" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="U46" s="26"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="15" t="s">
-        <v>263</v>
-      </c>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="16" t="n">
-        <f aca="false">SUM(K5:K46)</f>
-        <v>41990.96</v>
-      </c>
-      <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-      <c r="N47" s="6"/>
-      <c r="O47" s="16" t="n">
-        <f aca="false">SUM(O5:O46)</f>
-        <v>56288.61</v>
-      </c>
-      <c r="P47" s="6"/>
-      <c r="Q47" s="6"/>
-      <c r="R47" s="6"/>
-      <c r="S47" s="16" t="n">
-        <f aca="false">SUM(S5:S46)</f>
-        <v>77710.51</v>
-      </c>
-      <c r="T47" s="6"/>
-      <c r="U47" s="6"/>
+    <row r="47" customFormat="false" ht="326.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="E47" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="F47" s="27" t="s">
+        <v>270</v>
+      </c>
+      <c r="G47" s="20" t="n">
+        <f aca="false">p_Kitchen_Contingency_Rate/100*((1)*275.5 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (p_Kitchen_Travel_Hours)*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*580 + (4 + ROUNDUP(1.1*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*33.35 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*26 + (1)*435 + (p_Kitchen_Appliances_Supplied)*1015 + (p_Kitchen_New_Flooring_Area)*5.8 + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0))*100 + (p_Kitchen_Light_Fixtures)*116 + (p_Kitchen_Recessed_Lights)*36.25 + (p_Kitchen_Under_Cabinet_Lighting)*435)</f>
+        <v>3359.2768</v>
+      </c>
+      <c r="H47" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="J47" s="23" t="n">
+        <f aca="false">H47*INDEX(MarkupVals,MATCH(I47,MarkupCodes,0))</f>
+        <v>1</v>
+      </c>
+      <c r="K47" s="24" t="n">
+        <f aca="false">G47*J47</f>
+        <v>3359.2768</v>
+      </c>
+      <c r="L47" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="N47" s="23" t="n">
+        <f aca="false">L47*INDEX(MarkupVals,MATCH(M47,MarkupCodes,0))</f>
+        <v>0</v>
+      </c>
+      <c r="O47" s="24" t="n">
+        <f aca="false">G47*N47</f>
+        <v>0</v>
+      </c>
+      <c r="P47" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="R47" s="23" t="n">
+        <f aca="false">P47*INDEX(MarkupVals,MATCH(Q47,MarkupCodes,0))</f>
+        <v>0</v>
+      </c>
+      <c r="S47" s="24" t="n">
+        <f aca="false">G47*R47</f>
+        <v>0</v>
+      </c>
+      <c r="T47" s="25"/>
+      <c r="U47" s="26" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="326.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="D48" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="E48" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="F48" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="G48" s="20" t="n">
+        <f aca="false">p_Kitchen_Contingency_Rate/100*((1)*275.5 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (p_Kitchen_Travel_Hours)*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*870 + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*104 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*45.5 + (1)*870 + (p_Kitchen_Appliances_Supplied)*2030 + (p_Kitchen_New_Flooring_Area)*7.25 + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0))*100 + (p_Kitchen_Light_Fixtures)*261 + (p_Kitchen_Recessed_Lights)*50.75 + (p_Kitchen_Under_Cabinet_Lighting)*725)</f>
+        <v>4503.0888</v>
+      </c>
+      <c r="H48" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="J48" s="23" t="n">
+        <f aca="false">H48*INDEX(MarkupVals,MATCH(I48,MarkupCodes,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K48" s="24" t="n">
+        <f aca="false">G48*J48</f>
+        <v>0</v>
+      </c>
+      <c r="L48" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="N48" s="23" t="n">
+        <f aca="false">L48*INDEX(MarkupVals,MATCH(M48,MarkupCodes,0))</f>
+        <v>1</v>
+      </c>
+      <c r="O48" s="24" t="n">
+        <f aca="false">G48*N48</f>
+        <v>4503.0888</v>
+      </c>
+      <c r="P48" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="R48" s="23" t="n">
+        <f aca="false">P48*INDEX(MarkupVals,MATCH(Q48,MarkupCodes,0))</f>
+        <v>0</v>
+      </c>
+      <c r="S48" s="24" t="n">
+        <f aca="false">G48*R48</f>
+        <v>0</v>
+      </c>
+      <c r="T48" s="25"/>
+      <c r="U48" s="26" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="315.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="E49" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="F49" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <f aca="false">p_Kitchen_Contingency_Rate/100*((1)*275.5 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (p_Kitchen_Travel_Hours)*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*1305 + (4 + ROUNDUP(1.5*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*159.9 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*156 + (1)*1450 + (p_Kitchen_Appliances_Supplied)*3335 + (p_Kitchen_New_Flooring_Area)*19.5 + (p_Kitchen_Light_Fixtures)*507.5 + (p_Kitchen_Recessed_Lights)*87 + (p_Kitchen_Under_Cabinet_Lighting)*1116.5)</f>
+        <v>6216.8408</v>
+      </c>
+      <c r="H49" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="J49" s="23" t="n">
+        <f aca="false">H49*INDEX(MarkupVals,MATCH(I49,MarkupCodes,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K49" s="24" t="n">
+        <f aca="false">G49*J49</f>
+        <v>0</v>
+      </c>
+      <c r="L49" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="N49" s="23" t="n">
+        <f aca="false">L49*INDEX(MarkupVals,MATCH(M49,MarkupCodes,0))</f>
+        <v>0</v>
+      </c>
+      <c r="O49" s="24" t="n">
+        <f aca="false">G49*N49</f>
+        <v>0</v>
+      </c>
+      <c r="P49" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q49" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="R49" s="23" t="n">
+        <f aca="false">P49*INDEX(MarkupVals,MATCH(Q49,MarkupCodes,0))</f>
+        <v>1</v>
+      </c>
+      <c r="S49" s="24" t="n">
+        <f aca="false">G49*R49</f>
+        <v>6216.8408</v>
+      </c>
+      <c r="T49" s="25"/>
+      <c r="U49" s="26" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6"/>
+      <c r="K50" s="16" t="n">
+        <f aca="false">SUM(K5:K49)</f>
+        <v>45350.2368</v>
+      </c>
+      <c r="L50" s="6"/>
+      <c r="M50" s="6"/>
+      <c r="N50" s="6"/>
+      <c r="O50" s="16" t="n">
+        <f aca="false">SUM(O5:O49)</f>
+        <v>60791.6988</v>
+      </c>
+      <c r="P50" s="6"/>
+      <c r="Q50" s="6"/>
+      <c r="R50" s="6"/>
+      <c r="S50" s="16" t="n">
+        <f aca="false">SUM(S5:S49)</f>
+        <v>83927.3508</v>
+      </c>
+      <c r="T50" s="6"/>
+      <c r="U50" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5535,7 +5835,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -5547,7 +5847,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>264</v>
+        <v>278</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -5556,7 +5856,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>265</v>
+        <v>279</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -5572,377 +5872,392 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>269</v>
+        <v>283</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>270</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C5" s="28" t="n">
         <v>180</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>24</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>274</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="27" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="28" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>278</v>
+        <v>292</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>4</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E16" s="28" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C17" s="28" t="n">
         <v>2</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C18" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C19" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>281</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C20" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>282</v>
+        <v>296</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="27" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C21" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E21" s="28" t="s">
-        <v>283</v>
+        <v>297</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C22" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C23" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E23" s="28" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="27" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C24" s="28" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>271</v>
+        <v>285</v>
       </c>
       <c r="C25" s="28" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>163</v>
-      </c>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>285</v>
+      </c>
+      <c r="C26" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="E26" s="28"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5960,7 +6275,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -5971,7 +6286,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -5985,119 +6300,147 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>289</v>
+        <v>303</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="C4" s="29" t="n">
-        <f aca="false">C10/C9</f>
+        <f aca="false">C12/C11</f>
         <v>1.81818181818182</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="C5" s="30" t="n">
         <v>1.45</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="C6" s="30" t="n">
         <v>1.3</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="C7" s="30" t="n">
         <v>1.45</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="A8" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="C8" s="30" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="31" t="n">
+      <c r="A9" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="31" t="n">
         <v>55</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>300</v>
-      </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="31" t="n">
-        <v>100</v>
-      </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="D11" s="7" t="s">
+        <v>317</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>301</v>
+        <v>318</v>
       </c>
       <c r="B12" s="6"/>
-      <c r="C12" s="32" t="n">
+      <c r="C12" s="31" t="n">
+        <v>100</v>
+      </c>
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>302</v>
+      <c r="D14" s="7" t="s">
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -6126,7 +6469,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -6162,7 +6505,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -6198,7 +6541,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>305</v>
+        <v>323</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -6268,7 +6611,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -6304,108 +6647,108 @@
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>311</v>
+        <v>329</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>313</v>
+        <v>331</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>316</v>
+        <v>334</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O6" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="P6" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T6" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V6" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="W6" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="X6" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Z6" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="AA6" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AB6" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AC6" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AD6" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AE6" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AF6" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>319</v>
+        <v>337</v>
       </c>
       <c r="C7" s="33" t="n">
         <v>98048.85</v>
@@ -6502,10 +6845,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>319</v>
+        <v>337</v>
       </c>
       <c r="C8" s="33" t="n">
         <v>91172.79</v>
@@ -6636,7 +6979,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>321</v>
+        <v>339</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -6672,19 +7015,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>322</v>
+        <v>340</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>324</v>
+        <v>342</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>325</v>
+        <v>343</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>326</v>
+        <v>344</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -6716,10 +7059,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="C12" s="35" t="n">
         <v>870</v>
@@ -6761,10 +7104,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="C13" s="35" t="n">
         <v>1178</v>
@@ -6806,10 +7149,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="C14" s="35" t="n">
         <v>33.75</v>
@@ -6851,10 +7194,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="C15" s="35" t="n">
         <v>174</v>
@@ -6896,10 +7239,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="C16" s="35" t="n">
         <v>169.34</v>
@@ -6941,10 +7284,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="C17" s="35" t="n">
         <v>40</v>
@@ -6986,10 +7329,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="C18" s="35" t="n">
         <v>72</v>
@@ -7065,7 +7408,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -7101,7 +7444,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>

</xml_diff>

<commit_message>
Price permits by jurisdiction and travel by service zone
Answers the last three open items from 28 Sep 2026:

- Permit: each template has a Permit Fee parameter the estimator sets
  from DB's permit bills by jurisdiction (table on every workbook's Rates
  tab and in the proposal §9). Defaults stay at each type's old amount.
- Travel: a Service Zone parameter replaces typed-in travel hours. Travel
  is person-days x 0.5 h (Zone 2) or 1.25 h (Zone 3), from DB's own
  Service Call zone charges; Zone 1 adds none; Extended is quoted.
- Kitchen appliances are not supplied by default.

The intake sheets get a service-zone and permit row and still print on
two pages. Examples and calibration results are unchanged except the
Extended-zone bathroom (261280), which now gets 36 formula travel hours
against its estimated 30.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ch22kiCEY7KwpDM4Ye9Kr8
</commit_message>
<xml_diff>
--- a/docs/ballpark/kitchen-ballpark-template.xlsx
+++ b/docs/ballpark/kitchen-ballpark-template.xlsx
@@ -36,9 +36,10 @@
     <definedName function="false" hidden="false" name="p_Kitchen_Island_Length" vbProcedure="false">Calculator!$B$8</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Light_Fixtures" vbProcedure="false">Calculator!$B$15</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_New_Flooring_Area" vbProcedure="false">Calculator!$B$14</definedName>
+    <definedName function="false" hidden="false" name="p_Kitchen_Permit_Fee" vbProcedure="false">Calculator!$B$27</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Recessed_Lights" vbProcedure="false">Calculator!$B$16</definedName>
+    <definedName function="false" hidden="false" name="p_Kitchen_Service_Zone" vbProcedure="false">Calculator!$B$25</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Subfloor_Repair_Area" vbProcedure="false">Calculator!$B$20</definedName>
-    <definedName function="false" hidden="false" name="p_Kitchen_Travel_Hours" vbProcedure="false">Calculator!$B$25</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Under_Cabinet_Lighting" vbProcedure="false">Calculator!$B$18</definedName>
     <definedName function="false" hidden="false" name="p_Kitchen_Walls_Moved" vbProcedure="false">Calculator!$B$19</definedName>
     <definedName function="false" hidden="false" name="RangePct" vbProcedure="false">Rates!$C$14</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="389">
   <si>
     <t xml:space="preserve">Kitchen Ballpark Template — DRAFT for review</t>
   </si>
@@ -220,7 +221,7 @@
     <t xml:space="preserve">Kitchen Appliances Supplied</t>
   </si>
   <si>
-    <t xml:space="preserve">Appliances DB buys for the customer</t>
+    <t xml:space="preserve">Appliances DB buys for the customer. DB does not supply appliances by default: 0 unless the customer asks DB to buy them</t>
   </si>
   <si>
     <t xml:space="preserve">{Kitchen Appliances Supplied}</t>
@@ -376,13 +377,13 @@
     <t xml:space="preserve">{Kitchen Dumpster Loads}</t>
   </si>
   <si>
-    <t xml:space="preserve">Kitchen Travel Hours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crew travel hours for jobs past the standard service zone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{Kitchen Travel Hours}</t>
+    <t xml:space="preserve">Kitchen Service Zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service Zone from the job in JobTread: 1 (within ~15 mi), 2 (~15-30 mi), 3 (~30-50 mi). Zone 1 adds no travel. Extended (over 50 mi) is quoted by hand: enter 4 as a floor and flag it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Service Zone}</t>
   </si>
   <si>
     <t xml:space="preserve">Kitchen Contingency Rate</t>
@@ -394,6 +395,15 @@
     <t xml:space="preserve">{Kitchen Contingency Rate}</t>
   </si>
   <si>
+    <t xml:space="preserve">Kitchen Permit Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit fee DB pays the city or township, in dollars (cost), from the permit table on the Rates tab. The estimator sets it from the job address.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{Kitchen Permit Fee}</t>
+  </si>
+  <si>
     <t xml:space="preserve">JobTread build sheet: cost group "BALLPARK — Kitchen"</t>
   </si>
   <si>
@@ -475,45 +485,45 @@
     <t xml:space="preserve">Lump Sum</t>
   </si>
   <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantity is the permit fee in dollars at $1.00 each, so it can follow the jurisdiction: the estimator enters the fee from the permit table on the Rates tab as the Permit Fee parameter. Marked up like other costs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BALLPARK — Kitchen &gt; Phase 1 - General Requirements &gt; Project/Site Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Management (C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 + 4*{Kitchen Full Gut}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BALLPARK — Kitchen &gt; Phase 1 - General Requirements &gt; Site Preparation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Prep Material</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site Construction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each</t>
+  </si>
+  <si>
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kitchen permits on DB's two full kitchens were $275 and $287 price. Adjust per city.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BALLPARK — Kitchen &gt; Phase 1 - General Requirements &gt; Project/Site Management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Management (C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 + 4*{Kitchen Full Gut}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BALLPARK — Kitchen &gt; Phase 1 - General Requirements &gt; Site Preparation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site Prep Material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site Construction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each</t>
-  </si>
-  <si>
     <t xml:space="preserve">M</t>
   </si>
   <si>
@@ -565,6 +575,12 @@
     <t xml:space="preserve">Travel Related Costs</t>
   </si>
   <si>
+    <t xml:space="preserve">ceil(({Kitchen Service Zone} - 1)*({Kitchen Service Zone} + 2)/8*((4 + 4*{Kitchen Full Gut}) + (2) + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved}) + (2 + 2*{Kitchen Full Gut}) + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8)) + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated}) + (2*{Kitchen HVAC Work}) + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting}) + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15)) + (3 + ceil({Kitchen Floor Area}/20)) + (2*{Kitchen Appliances Installed}) + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors}) + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors}) + (4 + ceil(1.3*{Kitchen Cabinet Run})) + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000)))/8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel by the job's Service Zone (JobTread sets it from the address): hours = person-days x (z-1)(z+2)/8, which is 0, 0.5 and 1.25 h per person-day for Zones 1, 2 and 3. Those are DB's own Service Call zone charges ($85 / $115 / $155 cost) turned into travel time. Extended (over 50 mi) is quoted by hand; zone 4 gives 2.25 h per person-day as a floor.</t>
+  </si>
+  <si>
     <t xml:space="preserve">BALLPARK — Kitchen &gt; Phase 2 - Rough-In &gt; Framing Materials</t>
   </si>
   <si>
@@ -826,7 +842,7 @@
     <t xml:space="preserve">Appliance Allowance</t>
   </si>
   <si>
-    <t xml:space="preserve">Only appliances DB buys. Many customers supply their own; they still count toward install hours.</t>
+    <t xml:space="preserve">Only appliances DB buys. DB does not supply appliances by default (decided 28 Sep 2026): count them only when the customer asks. Appliances the customer buys still count toward install hours.</t>
   </si>
   <si>
     <t xml:space="preserve">Flooring Material</t>
@@ -865,7 +881,7 @@
     <t xml:space="preserve">Contingency</t>
   </si>
   <si>
-    <t xml:space="preserve">{Kitchen Contingency Rate}/100*((1)*275.5 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + ({Kitchen Travel Hours})*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*580 + (4 + ceil(1.1*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*33.35 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*26 + (1)*435 + ({Kitchen Appliances Supplied})*1015 + ({Kitchen New Flooring Area})*5.8 + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000))*100 + ({Kitchen Light Fixtures})*116 + ({Kitchen Recessed Lights})*36.25 + ({Kitchen Under-Cabinet Lighting})*435)</t>
+    <t xml:space="preserve">{Kitchen Contingency Rate}/100*(({Kitchen Permit Fee})*1.45 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + (ceil(({Kitchen Service Zone} - 1)*({Kitchen Service Zone} + 2)/8*((4 + 4*{Kitchen Full Gut}) + (2) + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved}) + (2 + 2*{Kitchen Full Gut}) + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8)) + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated}) + (2*{Kitchen HVAC Work}) + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting}) + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15)) + (3 + ceil({Kitchen Floor Area}/20)) + (2*{Kitchen Appliances Installed}) + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors}) + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors}) + (4 + ceil(1.3*{Kitchen Cabinet Run})) + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000)))/8))*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*580 + (4 + ceil(1.1*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*33.35 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*26 + (1)*435 + ({Kitchen Appliances Supplied})*1015 + ({Kitchen New Flooring Area})*5.8 + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000))*100 + ({Kitchen Light Fixtures})*116 + ({Kitchen Recessed Lights})*36.25 + ({Kitchen Under-Cabinet Lighting})*435)</t>
   </si>
   <si>
     <t xml:space="preserve">C</t>
@@ -877,13 +893,13 @@
     <t xml:space="preserve">Contingency — Better</t>
   </si>
   <si>
-    <t xml:space="preserve">{Kitchen Contingency Rate}/100*((1)*275.5 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + ({Kitchen Travel Hours})*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*870 + (4 + ceil(1.3*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*104 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*45.5 + (1)*870 + ({Kitchen Appliances Supplied})*2030 + ({Kitchen New Flooring Area})*7.25 + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000))*100 + ({Kitchen Light Fixtures})*261 + ({Kitchen Recessed Lights})*50.75 + ({Kitchen Under-Cabinet Lighting})*725)</t>
+    <t xml:space="preserve">{Kitchen Contingency Rate}/100*(({Kitchen Permit Fee})*1.45 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + (ceil(({Kitchen Service Zone} - 1)*({Kitchen Service Zone} + 2)/8*((4 + 4*{Kitchen Full Gut}) + (2) + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved}) + (2 + 2*{Kitchen Full Gut}) + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8)) + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated}) + (2*{Kitchen HVAC Work}) + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting}) + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15)) + (3 + ceil({Kitchen Floor Area}/20)) + (2*{Kitchen Appliances Installed}) + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors}) + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors}) + (4 + ceil(1.3*{Kitchen Cabinet Run})) + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000)))/8))*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*870 + (4 + ceil(1.3*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*104 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*45.5 + (1)*870 + ({Kitchen Appliances Supplied})*2030 + ({Kitchen New Flooring Area})*7.25 + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000))*100 + ({Kitchen Light Fixtures})*261 + ({Kitchen Recessed Lights})*50.75 + ({Kitchen Under-Cabinet Lighting})*725)</t>
   </si>
   <si>
     <t xml:space="preserve">Contingency — Best</t>
   </si>
   <si>
-    <t xml:space="preserve">{Kitchen Contingency Rate}/100*((1)*275.5 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + ({Kitchen Travel Hours})*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*1305 + (4 + ceil(1.5*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*159.9 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*156 + (1)*1450 + ({Kitchen Appliances Supplied})*3335 + ({Kitchen New Flooring Area})*19.5 + ({Kitchen Light Fixtures})*507.5 + ({Kitchen Recessed Lights})*87 + ({Kitchen Under-Cabinet Lighting})*1116.5)</t>
+    <t xml:space="preserve">{Kitchen Contingency Rate}/100*(({Kitchen Permit Fee})*1.45 + (4 + 4*{Kitchen Full Gut})*100 + (1)*217.5 + (2)*100 + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved})*100 + ({Kitchen Dumpster Loads})*450 + (2 + 2*{Kitchen Full Gut})*100 + (ceil(({Kitchen Service Zone} - 1)*({Kitchen Service Zone} + 2)/8*((4 + 4*{Kitchen Full Gut}) + (2) + (8 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15) + 6*{Kitchen Walls Moved}) + (2 + 2*{Kitchen Full Gut}) + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8)) + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated}) + (2*{Kitchen HVAC Work}) + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting}) + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15)) + (3 + ceil({Kitchen Floor Area}/20)) + (2*{Kitchen Appliances Installed}) + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors}) + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors}) + (4 + ceil(1.3*{Kitchen Cabinet Run})) + (ceil({Kitchen New Flooring Area}/20) + ceil({Kitchen New Flooring Area}/10000)))/8))*100 + ({Kitchen Full Gut} + 3*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/32))*217.5 + (4*{Kitchen Full Gut} + 8*{Kitchen Walls Moved} + ceil({Kitchen Subfloor Repair Area}/8))*100 + (1 + {Kitchen Fixtures Replaced} + 5*{Kitchen Fixtures Relocated})*145 + (3 + round(2.5*{Kitchen Fixtures Replaced}) + 4*{Kitchen Fixtures Relocated})*100 + ({Kitchen HVAC Work})*145 + (2*{Kitchen HVAC Work})*100 + ({Kitchen Floor Area})*3.7845 + (4 + {Kitchen Light Fixtures} + {Kitchen Recessed Lights} + 3*{Kitchen Circuits Added} + 3*{Kitchen Under-Cabinet Lighting})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*33.35 + (6 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/15))*100 + (1 + {Kitchen Full Gut})*166.75 + (3 + ceil({Kitchen Floor Area}/20))*100 + ({Kitchen New Flooring Area})*1.0875 + (ceil(2.5*{Kitchen Cabinet Run}))*14.5 + (2*{Kitchen Appliances Installed})*100 + ({Kitchen Interior Doors})*580 + ({Kitchen Exterior Doors})*1783.5 + (3*{Kitchen Interior Doors} + 8*{Kitchen Exterior Doors})*100 + (1 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/10))*29 + (2 + {Kitchen Full Gut}*ceil({Kitchen Floor Area}/12) + {Kitchen Interior Doors} + 2*{Kitchen Exterior Doors})*100 + ({Kitchen Cabinet Run})*1305 + (4 + ceil(1.5*{Kitchen Cabinet Run}))*100 + (2*{Kitchen Cabinet Run} + ceil(1.5*{Kitchen Island Length}))*159.9 + ({Kitchen Backsplash}*ceil(1.5*({Kitchen Cabinet Run} - {Kitchen Island Length})))*156 + (1)*1450 + ({Kitchen Appliances Supplied})*3335 + ({Kitchen New Flooring Area})*19.5 + ({Kitchen Light Fixtures})*507.5 + ({Kitchen Recessed Lights})*87 + ({Kitchen Under-Cabinet Lighting})*1116.5)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -913,46 +929,52 @@
     <t xml:space="preserve">Number</t>
   </si>
   <si>
-    <t xml:space="preserve">Demolition, Drywall Labor, Drywall Materials, Electrical Materials, Paint Labor, Trim Labor, Trim Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demolition, Drywall Labor, Drywall Materials, Final Clean, Framing/Sheathing Labor, Framing/Sheathing Materials, Paint Materials, Project Management (C), Trim Labor, Trim Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backsplash, Cabinet Knob/Pull, Cabinetry Labor, Cabinets, Countertops</t>
+    <t xml:space="preserve">Demolition, Drywall Labor, Drywall Materials, Electrical Materials, Paint Labor, Travel, Trim Labor, Trim Materials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demolition, Drywall Labor, Drywall Materials, Final Clean, Framing/Sheathing Labor, Framing/Sheathing Materials, Paint Materials, Project Management (C), Travel, Trim Labor, Trim Materials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backsplash, Cabinet Knob/Pull, Cabinetry Labor, Cabinets, Countertops, Travel</t>
   </si>
   <si>
     <t xml:space="preserve">Backsplash, Countertops</t>
   </si>
   <si>
-    <t xml:space="preserve">Plumbing Labor, Plumbing Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flooring - Misc. Material, Flooring Labor, Flooring Material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrical Labor, Light Fixture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrical Labor, Recessed Light</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrical Labor, Under-Cabinet Lighting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demolition, Framing/Sheathing Labor, Framing/Sheathing Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Framing/Sheathing Labor, Framing/Sheathing Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Door Labor, Interior Door, Trim Labor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Door Labor, Exterior Door &amp; Lockset, Trim Labor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HVAC Labor, HVAC Materials</t>
+    <t xml:space="preserve">Appliance Labor, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plumbing Labor, Plumbing Materials, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flooring - Misc. Material, Flooring Labor, Flooring Material, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical Labor, Light Fixture, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical Labor, Recessed Light, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical Labor, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical Labor, Travel, Under-Cabinet Lighting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demolition, Framing/Sheathing Labor, Framing/Sheathing Materials, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Framing/Sheathing Labor, Framing/Sheathing Materials, Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Door Labor, Interior Door, Travel, Trim Labor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Door Labor, Exterior Door &amp; Lockset, Travel, Trim Labor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HVAC Labor, HVAC Materials, Travel</t>
   </si>
   <si>
     <t xml:space="preserve">Markup by cost type</t>
@@ -1016,6 +1038,84 @@
   </si>
   <si>
     <t xml:space="preserve">Kitchens are quoted at ±20% until three have closed and the calibration is re-run (then ±15%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permit fees by jurisdiction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB's vendor bills for permits, last 6 months. Enter the job's fee as the Permit Fee parameter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jurisdiction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fee DB pays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Village of Convoy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City of Van Wert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$20 for the first $10K of project cost, plus $2 per additional $1K (paid $20–$122, average $36)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City of Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucas County</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$75.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Union Township</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pleasant Township Trustees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deitemeyer Brothers internal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$32–$40, average $36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel by service zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service Zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours per person-day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone 1 (within ~15 mi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone 2 (~15–30 mi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone 3 (~30–50 mi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extended (over 50 mi): quote by hand</t>
   </si>
   <si>
     <t xml:space="preserve">Checks against every kitchen DB has estimated since the move to JobTread</t>
@@ -1844,7 +1944,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -2420,7 +2520,7 @@
         <v>107</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>108</v>
@@ -2452,6 +2552,25 @@
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
       <c r="I26" s="6"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>190</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2485,7 +2604,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2510,7 +2629,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -2558,67 +2677,67 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="M4" s="8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="N4" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="O4" s="8" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="U4" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2626,61 +2745,61 @@
         <v>1</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="G5" s="20" t="n">
-        <f aca="false">1</f>
+        <f aca="false">p_Kitchen_Permit_Fee</f>
+        <v>190</v>
+      </c>
+      <c r="H5" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="21" t="n">
-        <v>190</v>
-      </c>
       <c r="I5" s="22" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J5" s="23" t="n">
         <f aca="false">H5*INDEX(MarkupVals,MATCH(I5,MarkupCodes,0))</f>
-        <v>275.5</v>
+        <v>1.45</v>
       </c>
       <c r="K5" s="24" t="n">
         <f aca="false">G5*J5</f>
         <v>275.5</v>
       </c>
       <c r="L5" s="21" t="n">
-        <v>190</v>
+        <v>1</v>
       </c>
       <c r="M5" s="22" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="N5" s="23" t="n">
         <f aca="false">L5*INDEX(MarkupVals,MATCH(M5,MarkupCodes,0))</f>
-        <v>275.5</v>
+        <v>1.45</v>
       </c>
       <c r="O5" s="24" t="n">
         <f aca="false">G5*N5</f>
         <v>275.5</v>
       </c>
       <c r="P5" s="21" t="n">
-        <v>190</v>
+        <v>1</v>
       </c>
       <c r="Q5" s="22" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="R5" s="23" t="n">
         <f aca="false">P5*INDEX(MarkupVals,MATCH(Q5,MarkupCodes,0))</f>
-        <v>275.5</v>
+        <v>1.45</v>
       </c>
       <c r="S5" s="24" t="n">
         <f aca="false">G5*R5</f>
@@ -2688,7 +2807,7 @@
       </c>
       <c r="T5" s="25"/>
       <c r="U5" s="26" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2696,19 +2815,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G6" s="20" t="n">
         <f aca="false">4 + 4*p_Kitchen_Full_Gut</f>
@@ -2719,7 +2838,7 @@
         <v>55</v>
       </c>
       <c r="I6" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">H6*INDEX(MarkupVals,MATCH(I6,MarkupCodes,0))</f>
@@ -2734,7 +2853,7 @@
         <v>55</v>
       </c>
       <c r="M6" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N6" s="23" t="n">
         <f aca="false">L6*INDEX(MarkupVals,MATCH(M6,MarkupCodes,0))</f>
@@ -2749,7 +2868,7 @@
         <v>55</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R6" s="23" t="n">
         <f aca="false">P6*INDEX(MarkupVals,MATCH(Q6,MarkupCodes,0))</f>
@@ -2767,19 +2886,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="G7" s="20" t="n">
         <f aca="false">1</f>
@@ -2789,7 +2908,7 @@
         <v>150</v>
       </c>
       <c r="I7" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J7" s="23" t="n">
         <f aca="false">H7*INDEX(MarkupVals,MATCH(I7,MarkupCodes,0))</f>
@@ -2803,7 +2922,7 @@
         <v>150</v>
       </c>
       <c r="M7" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N7" s="23" t="n">
         <f aca="false">L7*INDEX(MarkupVals,MATCH(M7,MarkupCodes,0))</f>
@@ -2817,7 +2936,7 @@
         <v>150</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R7" s="23" t="n">
         <f aca="false">P7*INDEX(MarkupVals,MATCH(Q7,MarkupCodes,0))</f>
@@ -2835,19 +2954,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="G8" s="20" t="n">
         <f aca="false">2</f>
@@ -2858,7 +2977,7 @@
         <v>55</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J8" s="23" t="n">
         <f aca="false">H8*INDEX(MarkupVals,MATCH(I8,MarkupCodes,0))</f>
@@ -2873,7 +2992,7 @@
         <v>55</v>
       </c>
       <c r="M8" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N8" s="23" t="n">
         <f aca="false">L8*INDEX(MarkupVals,MATCH(M8,MarkupCodes,0))</f>
@@ -2888,7 +3007,7 @@
         <v>55</v>
       </c>
       <c r="Q8" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R8" s="23" t="n">
         <f aca="false">P8*INDEX(MarkupVals,MATCH(Q8,MarkupCodes,0))</f>
@@ -2906,19 +3025,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G9" s="20" t="n">
         <f aca="false">8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved</f>
@@ -2929,7 +3048,7 @@
         <v>55</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J9" s="23" t="n">
         <f aca="false">H9*INDEX(MarkupVals,MATCH(I9,MarkupCodes,0))</f>
@@ -2944,7 +3063,7 @@
         <v>55</v>
       </c>
       <c r="M9" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N9" s="23" t="n">
         <f aca="false">L9*INDEX(MarkupVals,MATCH(M9,MarkupCodes,0))</f>
@@ -2959,7 +3078,7 @@
         <v>55</v>
       </c>
       <c r="Q9" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R9" s="23" t="n">
         <f aca="false">P9*INDEX(MarkupVals,MATCH(Q9,MarkupCodes,0))</f>
@@ -2971,7 +3090,7 @@
       </c>
       <c r="T9" s="25"/>
       <c r="U9" s="26" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2979,16 +3098,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F10" s="19" t="s">
         <v>106</v>
@@ -3001,7 +3120,7 @@
         <v>250</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J10" s="21" t="n">
         <v>450</v>
@@ -3014,7 +3133,7 @@
         <v>250</v>
       </c>
       <c r="M10" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N10" s="21" t="n">
         <v>450</v>
@@ -3027,7 +3146,7 @@
         <v>250</v>
       </c>
       <c r="Q10" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R10" s="21" t="n">
         <v>450</v>
@@ -3038,7 +3157,7 @@
       </c>
       <c r="T10" s="25"/>
       <c r="U10" s="26" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3046,19 +3165,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="G11" s="20" t="n">
         <f aca="false">2 + 2*p_Kitchen_Full_Gut</f>
@@ -3069,7 +3188,7 @@
         <v>55</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J11" s="23" t="n">
         <f aca="false">H11*INDEX(MarkupVals,MATCH(I11,MarkupCodes,0))</f>
@@ -3084,7 +3203,7 @@
         <v>55</v>
       </c>
       <c r="M11" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N11" s="23" t="n">
         <f aca="false">L11*INDEX(MarkupVals,MATCH(M11,MarkupCodes,0))</f>
@@ -3099,7 +3218,7 @@
         <v>55</v>
       </c>
       <c r="Q11" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R11" s="23" t="n">
         <f aca="false">P11*INDEX(MarkupVals,MATCH(Q11,MarkupCodes,0))</f>
@@ -3117,22 +3236,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>109</v>
+        <v>173</v>
       </c>
       <c r="G12" s="20" t="n">
-        <f aca="false">p_Kitchen_Travel_Hours</f>
+        <f aca="false">ROUNDUP((p_Kitchen_Service_Zone - 1)*(p_Kitchen_Service_Zone + 2)/8*((4 + 4*p_Kitchen_Full_Gut) + (2) + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved) + (2 + 2*p_Kitchen_Full_Gut) + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0)) + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated) + (2*p_Kitchen_HVAC_Work) + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting) + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0)) + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0)) + (2*p_Kitchen_Appliances_Installed) + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors) + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors) + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0)) + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)))/8,0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="23" t="n">
@@ -3140,7 +3259,7 @@
         <v>55</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">H12*INDEX(MarkupVals,MATCH(I12,MarkupCodes,0))</f>
@@ -3155,7 +3274,7 @@
         <v>55</v>
       </c>
       <c r="M12" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N12" s="23" t="n">
         <f aca="false">L12*INDEX(MarkupVals,MATCH(M12,MarkupCodes,0))</f>
@@ -3170,7 +3289,7 @@
         <v>55</v>
       </c>
       <c r="Q12" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R12" s="23" t="n">
         <f aca="false">P12*INDEX(MarkupVals,MATCH(Q12,MarkupCodes,0))</f>
@@ -3181,26 +3300,28 @@
         <v>0</v>
       </c>
       <c r="T12" s="25"/>
-      <c r="U12" s="26"/>
+      <c r="U12" s="26" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="G13" s="20" t="n">
         <f aca="false">p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0)</f>
@@ -3210,7 +3331,7 @@
         <v>150</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J13" s="23" t="n">
         <f aca="false">H13*INDEX(MarkupVals,MATCH(I13,MarkupCodes,0))</f>
@@ -3224,7 +3345,7 @@
         <v>150</v>
       </c>
       <c r="M13" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N13" s="23" t="n">
         <f aca="false">L13*INDEX(MarkupVals,MATCH(M13,MarkupCodes,0))</f>
@@ -3238,7 +3359,7 @@
         <v>150</v>
       </c>
       <c r="Q13" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R13" s="23" t="n">
         <f aca="false">P13*INDEX(MarkupVals,MATCH(Q13,MarkupCodes,0))</f>
@@ -3256,19 +3377,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="G14" s="20" t="n">
         <f aca="false">4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0)</f>
@@ -3279,7 +3400,7 @@
         <v>55</v>
       </c>
       <c r="I14" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J14" s="23" t="n">
         <f aca="false">H14*INDEX(MarkupVals,MATCH(I14,MarkupCodes,0))</f>
@@ -3294,7 +3415,7 @@
         <v>55</v>
       </c>
       <c r="M14" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N14" s="23" t="n">
         <f aca="false">L14*INDEX(MarkupVals,MATCH(M14,MarkupCodes,0))</f>
@@ -3309,7 +3430,7 @@
         <v>55</v>
       </c>
       <c r="Q14" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R14" s="23" t="n">
         <f aca="false">P14*INDEX(MarkupVals,MATCH(Q14,MarkupCodes,0))</f>
@@ -3327,19 +3448,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="G15" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated</f>
@@ -3349,7 +3470,7 @@
         <v>100</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J15" s="23" t="n">
         <f aca="false">H15*INDEX(MarkupVals,MATCH(I15,MarkupCodes,0))</f>
@@ -3363,7 +3484,7 @@
         <v>100</v>
       </c>
       <c r="M15" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N15" s="23" t="n">
         <f aca="false">L15*INDEX(MarkupVals,MATCH(M15,MarkupCodes,0))</f>
@@ -3377,7 +3498,7 @@
         <v>100</v>
       </c>
       <c r="Q15" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R15" s="23" t="n">
         <f aca="false">P15*INDEX(MarkupVals,MATCH(Q15,MarkupCodes,0))</f>
@@ -3389,7 +3510,7 @@
       </c>
       <c r="T15" s="25"/>
       <c r="U15" s="26" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3397,19 +3518,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="G16" s="20" t="n">
         <f aca="false">3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated</f>
@@ -3420,7 +3541,7 @@
         <v>55</v>
       </c>
       <c r="I16" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J16" s="23" t="n">
         <f aca="false">H16*INDEX(MarkupVals,MATCH(I16,MarkupCodes,0))</f>
@@ -3435,7 +3556,7 @@
         <v>55</v>
       </c>
       <c r="M16" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N16" s="23" t="n">
         <f aca="false">L16*INDEX(MarkupVals,MATCH(M16,MarkupCodes,0))</f>
@@ -3450,7 +3571,7 @@
         <v>55</v>
       </c>
       <c r="Q16" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R16" s="23" t="n">
         <f aca="false">P16*INDEX(MarkupVals,MATCH(Q16,MarkupCodes,0))</f>
@@ -3468,16 +3589,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C17" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="D17" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>179</v>
-      </c>
       <c r="E17" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>103</v>
@@ -3490,7 +3611,7 @@
         <v>100</v>
       </c>
       <c r="I17" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J17" s="23" t="n">
         <f aca="false">H17*INDEX(MarkupVals,MATCH(I17,MarkupCodes,0))</f>
@@ -3504,7 +3625,7 @@
         <v>100</v>
       </c>
       <c r="M17" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N17" s="23" t="n">
         <f aca="false">L17*INDEX(MarkupVals,MATCH(M17,MarkupCodes,0))</f>
@@ -3518,7 +3639,7 @@
         <v>100</v>
       </c>
       <c r="Q17" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R17" s="23" t="n">
         <f aca="false">P17*INDEX(MarkupVals,MATCH(Q17,MarkupCodes,0))</f>
@@ -3536,19 +3657,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="G18" s="20" t="n">
         <f aca="false">2*p_Kitchen_HVAC_Work</f>
@@ -3559,7 +3680,7 @@
         <v>55</v>
       </c>
       <c r="I18" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J18" s="23" t="n">
         <f aca="false">H18*INDEX(MarkupVals,MATCH(I18,MarkupCodes,0))</f>
@@ -3574,7 +3695,7 @@
         <v>55</v>
       </c>
       <c r="M18" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N18" s="23" t="n">
         <f aca="false">L18*INDEX(MarkupVals,MATCH(M18,MarkupCodes,0))</f>
@@ -3589,7 +3710,7 @@
         <v>55</v>
       </c>
       <c r="Q18" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R18" s="23" t="n">
         <f aca="false">P18*INDEX(MarkupVals,MATCH(Q18,MarkupCodes,0))</f>
@@ -3607,16 +3728,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="F19" s="19" t="s">
         <v>36</v>
@@ -3629,7 +3750,7 @@
         <v>2.61</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J19" s="23" t="n">
         <f aca="false">H19*INDEX(MarkupVals,MATCH(I19,MarkupCodes,0))</f>
@@ -3643,7 +3764,7 @@
         <v>2.61</v>
       </c>
       <c r="M19" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N19" s="23" t="n">
         <f aca="false">L19*INDEX(MarkupVals,MATCH(M19,MarkupCodes,0))</f>
@@ -3657,7 +3778,7 @@
         <v>2.61</v>
       </c>
       <c r="Q19" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R19" s="23" t="n">
         <f aca="false">P19*INDEX(MarkupVals,MATCH(Q19,MarkupCodes,0))</f>
@@ -3669,7 +3790,7 @@
       </c>
       <c r="T19" s="25"/>
       <c r="U19" s="26" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3677,19 +3798,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G20" s="20" t="n">
         <f aca="false">4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting</f>
@@ -3700,7 +3821,7 @@
         <v>55</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J20" s="23" t="n">
         <f aca="false">H20*INDEX(MarkupVals,MATCH(I20,MarkupCodes,0))</f>
@@ -3715,7 +3836,7 @@
         <v>55</v>
       </c>
       <c r="M20" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N20" s="23" t="n">
         <f aca="false">L20*INDEX(MarkupVals,MATCH(M20,MarkupCodes,0))</f>
@@ -3730,7 +3851,7 @@
         <v>55</v>
       </c>
       <c r="Q20" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R20" s="23" t="n">
         <f aca="false">P20*INDEX(MarkupVals,MATCH(Q20,MarkupCodes,0))</f>
@@ -3748,19 +3869,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="G21" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0)</f>
@@ -3770,7 +3891,7 @@
         <v>23</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J21" s="23" t="n">
         <f aca="false">H21*INDEX(MarkupVals,MATCH(I21,MarkupCodes,0))</f>
@@ -3784,7 +3905,7 @@
         <v>23</v>
       </c>
       <c r="M21" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N21" s="23" t="n">
         <f aca="false">L21*INDEX(MarkupVals,MATCH(M21,MarkupCodes,0))</f>
@@ -3798,7 +3919,7 @@
         <v>23</v>
       </c>
       <c r="Q21" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R21" s="23" t="n">
         <f aca="false">P21*INDEX(MarkupVals,MATCH(Q21,MarkupCodes,0))</f>
@@ -3810,7 +3931,7 @@
       </c>
       <c r="T21" s="25"/>
       <c r="U21" s="26" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3818,19 +3939,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="G22" s="20" t="n">
         <f aca="false">6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0)</f>
@@ -3841,7 +3962,7 @@
         <v>55</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J22" s="23" t="n">
         <f aca="false">H22*INDEX(MarkupVals,MATCH(I22,MarkupCodes,0))</f>
@@ -3856,7 +3977,7 @@
         <v>55</v>
       </c>
       <c r="M22" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N22" s="23" t="n">
         <f aca="false">L22*INDEX(MarkupVals,MATCH(M22,MarkupCodes,0))</f>
@@ -3871,7 +3992,7 @@
         <v>55</v>
       </c>
       <c r="Q22" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R22" s="23" t="n">
         <f aca="false">P22*INDEX(MarkupVals,MATCH(Q22,MarkupCodes,0))</f>
@@ -3889,19 +4010,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Full_Gut</f>
@@ -3911,7 +4032,7 @@
         <v>115</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J23" s="23" t="n">
         <f aca="false">H23*INDEX(MarkupVals,MATCH(I23,MarkupCodes,0))</f>
@@ -3925,7 +4046,7 @@
         <v>115</v>
       </c>
       <c r="M23" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N23" s="23" t="n">
         <f aca="false">L23*INDEX(MarkupVals,MATCH(M23,MarkupCodes,0))</f>
@@ -3939,7 +4060,7 @@
         <v>115</v>
       </c>
       <c r="Q23" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R23" s="23" t="n">
         <f aca="false">P23*INDEX(MarkupVals,MATCH(Q23,MarkupCodes,0))</f>
@@ -3957,19 +4078,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="G24" s="20" t="n">
         <f aca="false">3 + ROUNDUP(p_Kitchen_Floor_Area/20,0)</f>
@@ -3980,7 +4101,7 @@
         <v>55</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J24" s="23" t="n">
         <f aca="false">H24*INDEX(MarkupVals,MATCH(I24,MarkupCodes,0))</f>
@@ -3995,7 +4116,7 @@
         <v>55</v>
       </c>
       <c r="M24" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N24" s="23" t="n">
         <f aca="false">L24*INDEX(MarkupVals,MATCH(M24,MarkupCodes,0))</f>
@@ -4010,7 +4131,7 @@
         <v>55</v>
       </c>
       <c r="Q24" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R24" s="23" t="n">
         <f aca="false">P24*INDEX(MarkupVals,MATCH(Q24,MarkupCodes,0))</f>
@@ -4028,16 +4149,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="F25" s="19" t="s">
         <v>71</v>
@@ -4050,7 +4171,7 @@
         <v>0.75</v>
       </c>
       <c r="I25" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J25" s="23" t="n">
         <f aca="false">H25*INDEX(MarkupVals,MATCH(I25,MarkupCodes,0))</f>
@@ -4064,7 +4185,7 @@
         <v>0.75</v>
       </c>
       <c r="M25" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N25" s="23" t="n">
         <f aca="false">L25*INDEX(MarkupVals,MATCH(M25,MarkupCodes,0))</f>
@@ -4078,7 +4199,7 @@
         <v>0.75</v>
       </c>
       <c r="Q25" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R25" s="23" t="n">
         <f aca="false">P25*INDEX(MarkupVals,MATCH(Q25,MarkupCodes,0))</f>
@@ -4096,19 +4217,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="G26" s="20" t="n">
         <f aca="false">ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0)</f>
@@ -4118,7 +4239,7 @@
         <v>10</v>
       </c>
       <c r="I26" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J26" s="23" t="n">
         <f aca="false">H26*INDEX(MarkupVals,MATCH(I26,MarkupCodes,0))</f>
@@ -4132,7 +4253,7 @@
         <v>10</v>
       </c>
       <c r="M26" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N26" s="23" t="n">
         <f aca="false">L26*INDEX(MarkupVals,MATCH(M26,MarkupCodes,0))</f>
@@ -4146,7 +4267,7 @@
         <v>10</v>
       </c>
       <c r="Q26" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R26" s="23" t="n">
         <f aca="false">P26*INDEX(MarkupVals,MATCH(Q26,MarkupCodes,0))</f>
@@ -4164,19 +4285,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="G27" s="20" t="n">
         <f aca="false">2*p_Kitchen_Appliances_Installed</f>
@@ -4187,7 +4308,7 @@
         <v>55</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J27" s="23" t="n">
         <f aca="false">H27*INDEX(MarkupVals,MATCH(I27,MarkupCodes,0))</f>
@@ -4202,7 +4323,7 @@
         <v>55</v>
       </c>
       <c r="M27" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N27" s="23" t="n">
         <f aca="false">L27*INDEX(MarkupVals,MATCH(M27,MarkupCodes,0))</f>
@@ -4217,7 +4338,7 @@
         <v>55</v>
       </c>
       <c r="Q27" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R27" s="23" t="n">
         <f aca="false">P27*INDEX(MarkupVals,MATCH(Q27,MarkupCodes,0))</f>
@@ -4229,7 +4350,7 @@
       </c>
       <c r="T27" s="25"/>
       <c r="U27" s="26" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4237,16 +4358,16 @@
         <v>24</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F28" s="19" t="s">
         <v>97</v>
@@ -4259,7 +4380,7 @@
         <v>400</v>
       </c>
       <c r="I28" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J28" s="23" t="n">
         <f aca="false">H28*INDEX(MarkupVals,MATCH(I28,MarkupCodes,0))</f>
@@ -4273,7 +4394,7 @@
         <v>400</v>
       </c>
       <c r="M28" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N28" s="23" t="n">
         <f aca="false">L28*INDEX(MarkupVals,MATCH(M28,MarkupCodes,0))</f>
@@ -4287,7 +4408,7 @@
         <v>400</v>
       </c>
       <c r="Q28" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R28" s="23" t="n">
         <f aca="false">P28*INDEX(MarkupVals,MATCH(Q28,MarkupCodes,0))</f>
@@ -4305,16 +4426,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F29" s="19" t="s">
         <v>100</v>
@@ -4327,7 +4448,7 @@
         <v>1230</v>
       </c>
       <c r="I29" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J29" s="23" t="n">
         <f aca="false">H29*INDEX(MarkupVals,MATCH(I29,MarkupCodes,0))</f>
@@ -4341,7 +4462,7 @@
         <v>1230</v>
       </c>
       <c r="M29" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N29" s="23" t="n">
         <f aca="false">L29*INDEX(MarkupVals,MATCH(M29,MarkupCodes,0))</f>
@@ -4355,7 +4476,7 @@
         <v>1230</v>
       </c>
       <c r="Q29" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R29" s="23" t="n">
         <f aca="false">P29*INDEX(MarkupVals,MATCH(Q29,MarkupCodes,0))</f>
@@ -4367,7 +4488,7 @@
       </c>
       <c r="T29" s="25"/>
       <c r="U29" s="26" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4375,19 +4496,19 @@
         <v>26</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="G30" s="20" t="n">
         <f aca="false">3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors</f>
@@ -4398,7 +4519,7 @@
         <v>55</v>
       </c>
       <c r="I30" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J30" s="23" t="n">
         <f aca="false">H30*INDEX(MarkupVals,MATCH(I30,MarkupCodes,0))</f>
@@ -4413,7 +4534,7 @@
         <v>55</v>
       </c>
       <c r="M30" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N30" s="23" t="n">
         <f aca="false">L30*INDEX(MarkupVals,MATCH(M30,MarkupCodes,0))</f>
@@ -4428,7 +4549,7 @@
         <v>55</v>
       </c>
       <c r="Q30" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R30" s="23" t="n">
         <f aca="false">P30*INDEX(MarkupVals,MATCH(Q30,MarkupCodes,0))</f>
@@ -4446,19 +4567,19 @@
         <v>27</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="G31" s="20" t="n">
         <f aca="false">1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0)</f>
@@ -4468,7 +4589,7 @@
         <v>20</v>
       </c>
       <c r="I31" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J31" s="23" t="n">
         <f aca="false">H31*INDEX(MarkupVals,MATCH(I31,MarkupCodes,0))</f>
@@ -4482,7 +4603,7 @@
         <v>20</v>
       </c>
       <c r="M31" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N31" s="23" t="n">
         <f aca="false">L31*INDEX(MarkupVals,MATCH(M31,MarkupCodes,0))</f>
@@ -4496,7 +4617,7 @@
         <v>20</v>
       </c>
       <c r="Q31" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R31" s="23" t="n">
         <f aca="false">P31*INDEX(MarkupVals,MATCH(Q31,MarkupCodes,0))</f>
@@ -4514,19 +4635,19 @@
         <v>28</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="G32" s="20" t="n">
         <f aca="false">2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors</f>
@@ -4537,7 +4658,7 @@
         <v>55</v>
       </c>
       <c r="I32" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J32" s="23" t="n">
         <f aca="false">H32*INDEX(MarkupVals,MATCH(I32,MarkupCodes,0))</f>
@@ -4552,7 +4673,7 @@
         <v>55</v>
       </c>
       <c r="M32" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N32" s="23" t="n">
         <f aca="false">L32*INDEX(MarkupVals,MATCH(M32,MarkupCodes,0))</f>
@@ -4567,7 +4688,7 @@
         <v>55</v>
       </c>
       <c r="Q32" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R32" s="23" t="n">
         <f aca="false">P32*INDEX(MarkupVals,MATCH(Q32,MarkupCodes,0))</f>
@@ -4585,16 +4706,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C33" s="18" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="F33" s="19" t="s">
         <v>44</v>
@@ -4607,7 +4728,7 @@
         <v>400</v>
       </c>
       <c r="I33" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J33" s="23" t="n">
         <f aca="false">H33*INDEX(MarkupVals,MATCH(I33,MarkupCodes,0))</f>
@@ -4621,7 +4742,7 @@
         <v>600</v>
       </c>
       <c r="M33" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N33" s="23" t="n">
         <f aca="false">L33*INDEX(MarkupVals,MATCH(M33,MarkupCodes,0))</f>
@@ -4635,7 +4756,7 @@
         <v>900</v>
       </c>
       <c r="Q33" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R33" s="23" t="n">
         <f aca="false">P33*INDEX(MarkupVals,MATCH(Q33,MarkupCodes,0))</f>
@@ -4646,10 +4767,10 @@
         <v>33930</v>
       </c>
       <c r="T33" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U33" s="26" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4657,19 +4778,19 @@
         <v>30</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G34" s="20" t="n">
         <f aca="false">4 + ROUNDUP(1.1*p_Kitchen_Cabinet_Run,0)</f>
@@ -4680,7 +4801,7 @@
         <v>55</v>
       </c>
       <c r="I34" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J34" s="23" t="n">
         <f aca="false">H34*INDEX(MarkupVals,MATCH(I34,MarkupCodes,0))</f>
@@ -4694,7 +4815,7 @@
         <v>0</v>
       </c>
       <c r="M34" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N34" s="23" t="n">
         <f aca="false">L34*INDEX(MarkupVals,MATCH(M34,MarkupCodes,0))</f>
@@ -4708,7 +4829,7 @@
         <v>0</v>
       </c>
       <c r="Q34" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R34" s="23" t="n">
         <f aca="false">P34*INDEX(MarkupVals,MATCH(Q34,MarkupCodes,0))</f>
@@ -4720,7 +4841,7 @@
       </c>
       <c r="T34" s="25"/>
       <c r="U34" s="26" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4728,19 +4849,19 @@
         <v>31</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="G35" s="20" t="n">
         <f aca="false">4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0)</f>
@@ -4750,7 +4871,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J35" s="23" t="n">
         <f aca="false">H35*INDEX(MarkupVals,MATCH(I35,MarkupCodes,0))</f>
@@ -4765,7 +4886,7 @@
         <v>55</v>
       </c>
       <c r="M35" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N35" s="23" t="n">
         <f aca="false">L35*INDEX(MarkupVals,MATCH(M35,MarkupCodes,0))</f>
@@ -4779,7 +4900,7 @@
         <v>0</v>
       </c>
       <c r="Q35" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R35" s="23" t="n">
         <f aca="false">P35*INDEX(MarkupVals,MATCH(Q35,MarkupCodes,0))</f>
@@ -4791,7 +4912,7 @@
       </c>
       <c r="T35" s="25"/>
       <c r="U35" s="26" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4799,19 +4920,19 @@
         <v>32</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="G36" s="20" t="n">
         <f aca="false">4 + ROUNDUP(1.5*p_Kitchen_Cabinet_Run,0)</f>
@@ -4821,7 +4942,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J36" s="23" t="n">
         <f aca="false">H36*INDEX(MarkupVals,MATCH(I36,MarkupCodes,0))</f>
@@ -4835,7 +4956,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N36" s="23" t="n">
         <f aca="false">L36*INDEX(MarkupVals,MATCH(M36,MarkupCodes,0))</f>
@@ -4850,7 +4971,7 @@
         <v>55</v>
       </c>
       <c r="Q36" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R36" s="23" t="n">
         <f aca="false">P36*INDEX(MarkupVals,MATCH(Q36,MarkupCodes,0))</f>
@@ -4862,7 +4983,7 @@
       </c>
       <c r="T36" s="25"/>
       <c r="U36" s="26" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4870,19 +4991,19 @@
         <v>33</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G37" s="20" t="n">
         <f aca="false">2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0)</f>
@@ -4892,7 +5013,7 @@
         <v>23</v>
       </c>
       <c r="I37" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J37" s="23" t="n">
         <f aca="false">H37*INDEX(MarkupVals,MATCH(I37,MarkupCodes,0))</f>
@@ -4906,7 +5027,7 @@
         <v>80</v>
       </c>
       <c r="M37" s="22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="N37" s="23" t="n">
         <f aca="false">L37*INDEX(MarkupVals,MATCH(M37,MarkupCodes,0))</f>
@@ -4920,7 +5041,7 @@
         <v>123</v>
       </c>
       <c r="Q37" s="22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R37" s="23" t="n">
         <f aca="false">P37*INDEX(MarkupVals,MATCH(Q37,MarkupCodes,0))</f>
@@ -4931,10 +5052,10 @@
         <v>9753.9</v>
       </c>
       <c r="T37" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U37" s="26" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4942,19 +5063,19 @@
         <v>34</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="G38" s="20" t="n">
         <f aca="false">p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0)</f>
@@ -4964,7 +5085,7 @@
         <v>20</v>
       </c>
       <c r="I38" s="22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="J38" s="23" t="n">
         <f aca="false">H38*INDEX(MarkupVals,MATCH(I38,MarkupCodes,0))</f>
@@ -4978,7 +5099,7 @@
         <v>35</v>
       </c>
       <c r="M38" s="22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="N38" s="23" t="n">
         <f aca="false">L38*INDEX(MarkupVals,MATCH(M38,MarkupCodes,0))</f>
@@ -4992,7 +5113,7 @@
         <v>120</v>
       </c>
       <c r="Q38" s="22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R38" s="23" t="n">
         <f aca="false">P38*INDEX(MarkupVals,MATCH(Q38,MarkupCodes,0))</f>
@@ -5003,10 +5124,10 @@
         <v>4680</v>
       </c>
       <c r="T38" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U38" s="26" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5014,19 +5135,19 @@
         <v>35</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="G39" s="20" t="n">
         <f aca="false">1</f>
@@ -5036,7 +5157,7 @@
         <v>300</v>
       </c>
       <c r="I39" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J39" s="23" t="n">
         <f aca="false">H39*INDEX(MarkupVals,MATCH(I39,MarkupCodes,0))</f>
@@ -5050,7 +5171,7 @@
         <v>600</v>
       </c>
       <c r="M39" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N39" s="23" t="n">
         <f aca="false">L39*INDEX(MarkupVals,MATCH(M39,MarkupCodes,0))</f>
@@ -5064,7 +5185,7 @@
         <v>1000</v>
       </c>
       <c r="Q39" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R39" s="23" t="n">
         <f aca="false">P39*INDEX(MarkupVals,MATCH(Q39,MarkupCodes,0))</f>
@@ -5075,7 +5196,7 @@
         <v>1450</v>
       </c>
       <c r="T39" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U39" s="26"/>
     </row>
@@ -5084,16 +5205,16 @@
         <v>36</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F40" s="19" t="s">
         <v>56</v>
@@ -5106,7 +5227,7 @@
         <v>700</v>
       </c>
       <c r="I40" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J40" s="23" t="n">
         <f aca="false">H40*INDEX(MarkupVals,MATCH(I40,MarkupCodes,0))</f>
@@ -5120,7 +5241,7 @@
         <v>1400</v>
       </c>
       <c r="M40" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N40" s="23" t="n">
         <f aca="false">L40*INDEX(MarkupVals,MATCH(M40,MarkupCodes,0))</f>
@@ -5134,7 +5255,7 @@
         <v>2300</v>
       </c>
       <c r="Q40" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R40" s="23" t="n">
         <f aca="false">P40*INDEX(MarkupVals,MATCH(Q40,MarkupCodes,0))</f>
@@ -5145,10 +5266,10 @@
         <v>0</v>
       </c>
       <c r="T40" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U40" s="26" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5156,16 +5277,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C41" s="18" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="F41" s="19" t="s">
         <v>71</v>
@@ -5178,7 +5299,7 @@
         <v>4</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J41" s="23" t="n">
         <f aca="false">H41*INDEX(MarkupVals,MATCH(I41,MarkupCodes,0))</f>
@@ -5192,7 +5313,7 @@
         <v>5</v>
       </c>
       <c r="M41" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N41" s="23" t="n">
         <f aca="false">L41*INDEX(MarkupVals,MATCH(M41,MarkupCodes,0))</f>
@@ -5206,7 +5327,7 @@
         <v>15</v>
       </c>
       <c r="Q41" s="22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="R41" s="23" t="n">
         <f aca="false">P41*INDEX(MarkupVals,MATCH(Q41,MarkupCodes,0))</f>
@@ -5217,10 +5338,10 @@
         <v>3510</v>
       </c>
       <c r="T41" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U41" s="26" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5228,19 +5349,19 @@
         <v>38</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D42" s="18" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G42" s="20" t="n">
         <f aca="false">ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)</f>
@@ -5251,7 +5372,7 @@
         <v>55</v>
       </c>
       <c r="I42" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J42" s="23" t="n">
         <f aca="false">H42*INDEX(MarkupVals,MATCH(I42,MarkupCodes,0))</f>
@@ -5265,7 +5386,7 @@
         <v>0</v>
       </c>
       <c r="M42" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N42" s="23" t="n">
         <f aca="false">L42*INDEX(MarkupVals,MATCH(M42,MarkupCodes,0))</f>
@@ -5279,7 +5400,7 @@
         <v>0</v>
       </c>
       <c r="Q42" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R42" s="23" t="n">
         <f aca="false">P42*INDEX(MarkupVals,MATCH(Q42,MarkupCodes,0))</f>
@@ -5291,7 +5412,7 @@
       </c>
       <c r="T42" s="25"/>
       <c r="U42" s="26" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5299,19 +5420,19 @@
         <v>39</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C43" s="18" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D43" s="18" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E43" s="18" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="G43" s="20" t="n">
         <f aca="false">ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)</f>
@@ -5321,7 +5442,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J43" s="23" t="n">
         <f aca="false">H43*INDEX(MarkupVals,MATCH(I43,MarkupCodes,0))</f>
@@ -5336,7 +5457,7 @@
         <v>55</v>
       </c>
       <c r="M43" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N43" s="23" t="n">
         <f aca="false">L43*INDEX(MarkupVals,MATCH(M43,MarkupCodes,0))</f>
@@ -5350,7 +5471,7 @@
         <v>0</v>
       </c>
       <c r="Q43" s="22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="R43" s="23" t="n">
         <f aca="false">P43*INDEX(MarkupVals,MATCH(Q43,MarkupCodes,0))</f>
@@ -5362,7 +5483,7 @@
       </c>
       <c r="T43" s="25"/>
       <c r="U43" s="26" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5370,16 +5491,16 @@
         <v>40</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D44" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F44" s="19" t="s">
         <v>75</v>
@@ -5392,7 +5513,7 @@
         <v>80</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J44" s="23" t="n">
         <f aca="false">H44*INDEX(MarkupVals,MATCH(I44,MarkupCodes,0))</f>
@@ -5406,7 +5527,7 @@
         <v>180</v>
       </c>
       <c r="M44" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N44" s="23" t="n">
         <f aca="false">L44*INDEX(MarkupVals,MATCH(M44,MarkupCodes,0))</f>
@@ -5420,7 +5541,7 @@
         <v>350</v>
       </c>
       <c r="Q44" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R44" s="23" t="n">
         <f aca="false">P44*INDEX(MarkupVals,MATCH(Q44,MarkupCodes,0))</f>
@@ -5431,7 +5552,7 @@
         <v>1015</v>
       </c>
       <c r="T44" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U44" s="26"/>
     </row>
@@ -5440,16 +5561,16 @@
         <v>41</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E45" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F45" s="19" t="s">
         <v>79</v>
@@ -5462,7 +5583,7 @@
         <v>25</v>
       </c>
       <c r="I45" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J45" s="23" t="n">
         <f aca="false">H45*INDEX(MarkupVals,MATCH(I45,MarkupCodes,0))</f>
@@ -5476,7 +5597,7 @@
         <v>35</v>
       </c>
       <c r="M45" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N45" s="23" t="n">
         <f aca="false">L45*INDEX(MarkupVals,MATCH(M45,MarkupCodes,0))</f>
@@ -5490,7 +5611,7 @@
         <v>60</v>
       </c>
       <c r="Q45" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R45" s="23" t="n">
         <f aca="false">P45*INDEX(MarkupVals,MATCH(Q45,MarkupCodes,0))</f>
@@ -5501,7 +5622,7 @@
         <v>522</v>
       </c>
       <c r="T45" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U45" s="26"/>
     </row>
@@ -5510,16 +5631,16 @@
         <v>42</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E46" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F46" s="19" t="s">
         <v>86</v>
@@ -5532,7 +5653,7 @@
         <v>300</v>
       </c>
       <c r="I46" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J46" s="23" t="n">
         <f aca="false">H46*INDEX(MarkupVals,MATCH(I46,MarkupCodes,0))</f>
@@ -5546,7 +5667,7 @@
         <v>500</v>
       </c>
       <c r="M46" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="N46" s="23" t="n">
         <f aca="false">L46*INDEX(MarkupVals,MATCH(M46,MarkupCodes,0))</f>
@@ -5560,7 +5681,7 @@
         <v>770</v>
       </c>
       <c r="Q46" s="22" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="R46" s="23" t="n">
         <f aca="false">P46*INDEX(MarkupVals,MATCH(Q46,MarkupCodes,0))</f>
@@ -5571,38 +5692,38 @@
         <v>1116.5</v>
       </c>
       <c r="T46" s="25" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="U46" s="26"/>
     </row>
-    <row r="47" customFormat="false" ht="326.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="482.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="n">
         <v>43</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C47" s="18" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E47" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F47" s="27" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="G47" s="20" t="n">
-        <f aca="false">p_Kitchen_Contingency_Rate/100*((1)*275.5 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (p_Kitchen_Travel_Hours)*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*580 + (4 + ROUNDUP(1.1*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*33.35 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*26 + (1)*435 + (p_Kitchen_Appliances_Supplied)*1015 + (p_Kitchen_New_Flooring_Area)*5.8 + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0))*100 + (p_Kitchen_Light_Fixtures)*116 + (p_Kitchen_Recessed_Lights)*36.25 + (p_Kitchen_Under_Cabinet_Lighting)*435)</f>
+        <f aca="false">p_Kitchen_Contingency_Rate/100*((p_Kitchen_Permit_Fee)*1.45 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (ROUNDUP((p_Kitchen_Service_Zone - 1)*(p_Kitchen_Service_Zone + 2)/8*((4 + 4*p_Kitchen_Full_Gut) + (2) + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved) + (2 + 2*p_Kitchen_Full_Gut) + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0)) + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated) + (2*p_Kitchen_HVAC_Work) + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting) + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0)) + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0)) + (2*p_Kitchen_Appliances_Installed) + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors) + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors) + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0)) + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)))/8,0))*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*580 + (4 + ROUNDUP(1.1*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*33.35 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*26 + (1)*435 + (p_Kitchen_Appliances_Supplied)*1015 + (p_Kitchen_New_Flooring_Area)*5.8 + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0))*100 + (p_Kitchen_Light_Fixtures)*116 + (p_Kitchen_Recessed_Lights)*36.25 + (p_Kitchen_Under_Cabinet_Lighting)*435)</f>
         <v>3359.2768</v>
       </c>
       <c r="H47" s="21" t="n">
         <v>1</v>
       </c>
       <c r="I47" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="J47" s="23" t="n">
         <f aca="false">H47*INDEX(MarkupVals,MATCH(I47,MarkupCodes,0))</f>
@@ -5616,7 +5737,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="N47" s="23" t="n">
         <f aca="false">L47*INDEX(MarkupVals,MATCH(M47,MarkupCodes,0))</f>
@@ -5630,7 +5751,7 @@
         <v>0</v>
       </c>
       <c r="Q47" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="R47" s="23" t="n">
         <f aca="false">P47*INDEX(MarkupVals,MATCH(Q47,MarkupCodes,0))</f>
@@ -5642,37 +5763,37 @@
       </c>
       <c r="T47" s="25"/>
       <c r="U47" s="26" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="326.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="482.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="n">
         <v>44</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C48" s="18" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D48" s="18" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E48" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F48" s="27" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="G48" s="20" t="n">
-        <f aca="false">p_Kitchen_Contingency_Rate/100*((1)*275.5 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (p_Kitchen_Travel_Hours)*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*870 + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*104 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*45.5 + (1)*870 + (p_Kitchen_Appliances_Supplied)*2030 + (p_Kitchen_New_Flooring_Area)*7.25 + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0))*100 + (p_Kitchen_Light_Fixtures)*261 + (p_Kitchen_Recessed_Lights)*50.75 + (p_Kitchen_Under_Cabinet_Lighting)*725)</f>
+        <f aca="false">p_Kitchen_Contingency_Rate/100*((p_Kitchen_Permit_Fee)*1.45 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (ROUNDUP((p_Kitchen_Service_Zone - 1)*(p_Kitchen_Service_Zone + 2)/8*((4 + 4*p_Kitchen_Full_Gut) + (2) + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved) + (2 + 2*p_Kitchen_Full_Gut) + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0)) + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated) + (2*p_Kitchen_HVAC_Work) + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting) + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0)) + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0)) + (2*p_Kitchen_Appliances_Installed) + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors) + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors) + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0)) + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)))/8,0))*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*870 + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*104 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*45.5 + (1)*870 + (p_Kitchen_Appliances_Supplied)*2030 + (p_Kitchen_New_Flooring_Area)*7.25 + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0))*100 + (p_Kitchen_Light_Fixtures)*261 + (p_Kitchen_Recessed_Lights)*50.75 + (p_Kitchen_Under_Cabinet_Lighting)*725)</f>
         <v>4503.0888</v>
       </c>
       <c r="H48" s="21" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="J48" s="23" t="n">
         <f aca="false">H48*INDEX(MarkupVals,MATCH(I48,MarkupCodes,0))</f>
@@ -5686,7 +5807,7 @@
         <v>1</v>
       </c>
       <c r="M48" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="N48" s="23" t="n">
         <f aca="false">L48*INDEX(MarkupVals,MATCH(M48,MarkupCodes,0))</f>
@@ -5700,7 +5821,7 @@
         <v>0</v>
       </c>
       <c r="Q48" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="R48" s="23" t="n">
         <f aca="false">P48*INDEX(MarkupVals,MATCH(Q48,MarkupCodes,0))</f>
@@ -5712,37 +5833,37 @@
       </c>
       <c r="T48" s="25"/>
       <c r="U48" s="26" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="315.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="472.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="n">
         <v>45</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C49" s="18" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E49" s="18" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F49" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <f aca="false">p_Kitchen_Contingency_Rate/100*((p_Kitchen_Permit_Fee)*1.45 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (ROUNDUP((p_Kitchen_Service_Zone - 1)*(p_Kitchen_Service_Zone + 2)/8*((4 + 4*p_Kitchen_Full_Gut) + (2) + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved) + (2 + 2*p_Kitchen_Full_Gut) + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0)) + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated) + (2*p_Kitchen_HVAC_Work) + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting) + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0)) + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0)) + (2*p_Kitchen_Appliances_Installed) + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors) + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors) + (4 + ROUNDUP(1.3*p_Kitchen_Cabinet_Run,0)) + (ROUNDUP(p_Kitchen_New_Flooring_Area/20,0) + ROUNDUP(p_Kitchen_New_Flooring_Area/10000,0)))/8,0))*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*1305 + (4 + ROUNDUP(1.5*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*159.9 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*156 + (1)*1450 + (p_Kitchen_Appliances_Supplied)*3335 + (p_Kitchen_New_Flooring_Area)*19.5 + (p_Kitchen_Light_Fixtures)*507.5 + (p_Kitchen_Recessed_Lights)*87 + (p_Kitchen_Under_Cabinet_Lighting)*1116.5)</f>
+        <v>6216.8408</v>
+      </c>
+      <c r="H49" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="22" t="s">
         <v>276</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <f aca="false">p_Kitchen_Contingency_Rate/100*((1)*275.5 + (4 + 4*p_Kitchen_Full_Gut)*100 + (1)*217.5 + (2)*100 + (8 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0) + 6*p_Kitchen_Walls_Moved)*100 + (p_Kitchen_Dumpster_Loads)*450 + (2 + 2*p_Kitchen_Full_Gut)*100 + (p_Kitchen_Travel_Hours)*100 + (p_Kitchen_Full_Gut + 3*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/32,0))*217.5 + (4*p_Kitchen_Full_Gut + 8*p_Kitchen_Walls_Moved + ROUNDUP(p_Kitchen_Subfloor_Repair_Area/8,0))*100 + (1 + p_Kitchen_Fixtures_Replaced + 5*p_Kitchen_Fixtures_Relocated)*145 + (3 + ROUND(2.5*p_Kitchen_Fixtures_Replaced,0) + 4*p_Kitchen_Fixtures_Relocated)*100 + (p_Kitchen_HVAC_Work)*145 + (2*p_Kitchen_HVAC_Work)*100 + (p_Kitchen_Floor_Area)*3.7845 + (4 + p_Kitchen_Light_Fixtures + p_Kitchen_Recessed_Lights + 3*p_Kitchen_Circuits_Added + 3*p_Kitchen_Under_Cabinet_Lighting)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*33.35 + (6 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/15,0))*100 + (1 + p_Kitchen_Full_Gut)*166.75 + (3 + ROUNDUP(p_Kitchen_Floor_Area/20,0))*100 + (p_Kitchen_New_Flooring_Area)*1.0875 + (ROUNDUP(2.5*p_Kitchen_Cabinet_Run,0))*14.5 + (2*p_Kitchen_Appliances_Installed)*100 + (p_Kitchen_Interior_Doors)*580 + (p_Kitchen_Exterior_Doors)*1783.5 + (3*p_Kitchen_Interior_Doors + 8*p_Kitchen_Exterior_Doors)*100 + (1 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/10,0))*29 + (2 + p_Kitchen_Full_Gut*ROUNDUP(p_Kitchen_Floor_Area/12,0) + p_Kitchen_Interior_Doors + 2*p_Kitchen_Exterior_Doors)*100 + (p_Kitchen_Cabinet_Run)*1305 + (4 + ROUNDUP(1.5*p_Kitchen_Cabinet_Run,0))*100 + (2*p_Kitchen_Cabinet_Run + ROUNDUP(1.5*p_Kitchen_Island_Length,0))*159.9 + (p_Kitchen_Backsplash*ROUNDUP(1.5*(p_Kitchen_Cabinet_Run - p_Kitchen_Island_Length),0))*156 + (1)*1450 + (p_Kitchen_Appliances_Supplied)*3335 + (p_Kitchen_New_Flooring_Area)*19.5 + (p_Kitchen_Light_Fixtures)*507.5 + (p_Kitchen_Recessed_Lights)*87 + (p_Kitchen_Under_Cabinet_Lighting)*1116.5)</f>
-        <v>6216.8408</v>
-      </c>
-      <c r="H49" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" s="22" t="s">
-        <v>271</v>
       </c>
       <c r="J49" s="23" t="n">
         <f aca="false">H49*INDEX(MarkupVals,MATCH(I49,MarkupCodes,0))</f>
@@ -5756,7 +5877,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="N49" s="23" t="n">
         <f aca="false">L49*INDEX(MarkupVals,MATCH(M49,MarkupCodes,0))</f>
@@ -5770,7 +5891,7 @@
         <v>1</v>
       </c>
       <c r="Q49" s="22" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="R49" s="23" t="n">
         <f aca="false">P49*INDEX(MarkupVals,MATCH(Q49,MarkupCodes,0))</f>
@@ -5782,14 +5903,14 @@
       </c>
       <c r="T49" s="25"/>
       <c r="U49" s="26" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="15" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
@@ -5835,7 +5956,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -5847,7 +5968,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -5856,7 +5977,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -5872,27 +5993,27 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
         <v>34</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C5" s="28" t="n">
         <v>180</v>
@@ -5901,7 +6022,7 @@
         <v>35</v>
       </c>
       <c r="E5" s="28" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5909,7 +6030,7 @@
         <v>38</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -5918,7 +6039,7 @@
         <v>39</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5926,7 +6047,7 @@
         <v>42</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>24</v>
@@ -5935,7 +6056,7 @@
         <v>43</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5943,7 +6064,7 @@
         <v>46</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -5952,7 +6073,7 @@
         <v>47</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5960,7 +6081,7 @@
         <v>50</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>1</v>
@@ -5969,15 +6090,15 @@
         <v>51</v>
       </c>
       <c r="E9" s="28" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
         <v>54</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>0</v>
@@ -5986,7 +6107,7 @@
         <v>55</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5994,7 +6115,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>4</v>
@@ -6003,7 +6124,7 @@
         <v>59</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>215</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6011,7 +6132,7 @@
         <v>62</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -6020,7 +6141,7 @@
         <v>63</v>
       </c>
       <c r="E12" s="28" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6028,7 +6149,7 @@
         <v>66</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -6037,7 +6158,7 @@
         <v>67</v>
       </c>
       <c r="E13" s="28" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6045,7 +6166,7 @@
         <v>69</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -6054,7 +6175,7 @@
         <v>70</v>
       </c>
       <c r="E14" s="28" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6062,7 +6183,7 @@
         <v>73</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>1</v>
@@ -6071,7 +6192,7 @@
         <v>74</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6079,7 +6200,7 @@
         <v>77</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>4</v>
@@ -6088,7 +6209,7 @@
         <v>78</v>
       </c>
       <c r="E16" s="28" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6096,7 +6217,7 @@
         <v>81</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C17" s="28" t="n">
         <v>2</v>
@@ -6105,7 +6226,7 @@
         <v>82</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>192</v>
+        <v>300</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6113,7 +6234,7 @@
         <v>84</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C18" s="28" t="n">
         <v>0</v>
@@ -6122,7 +6243,7 @@
         <v>85</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6130,7 +6251,7 @@
         <v>88</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C19" s="28" t="n">
         <v>0</v>
@@ -6139,7 +6260,7 @@
         <v>89</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6147,7 +6268,7 @@
         <v>92</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C20" s="28" t="n">
         <v>0</v>
@@ -6156,7 +6277,7 @@
         <v>93</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6164,7 +6285,7 @@
         <v>95</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C21" s="28" t="n">
         <v>0</v>
@@ -6173,7 +6294,7 @@
         <v>96</v>
       </c>
       <c r="E21" s="28" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6181,7 +6302,7 @@
         <v>98</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C22" s="28" t="n">
         <v>0</v>
@@ -6190,7 +6311,7 @@
         <v>99</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6198,7 +6319,7 @@
         <v>101</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C23" s="28" t="n">
         <v>0</v>
@@ -6207,7 +6328,7 @@
         <v>102</v>
       </c>
       <c r="E23" s="28" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6215,7 +6336,7 @@
         <v>104</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C24" s="28" t="n">
         <v>1</v>
@@ -6224,24 +6345,24 @@
         <v>105</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="s">
         <v>107</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C25" s="28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="28" t="s">
         <v>108</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6249,7 +6370,7 @@
         <v>110</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C26" s="28" t="n">
         <v>8</v>
@@ -6258,6 +6379,23 @@
         <v>111</v>
       </c>
       <c r="E26" s="28"/>
+    </row>
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>290</v>
+      </c>
+      <c r="C27" s="28" t="n">
+        <v>190</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="28" t="s">
+        <v>140</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6275,18 +6413,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -6300,101 +6438,101 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C4" s="29" t="n">
         <f aca="false">C12/C11</f>
         <v>1.81818181818182</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="C5" s="30" t="n">
         <v>1.45</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="C6" s="30" t="n">
         <v>1.3</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C7" s="30" t="n">
         <v>1.45</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C8" s="30" t="n">
         <v>1.45</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C9" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6405,19 +6543,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="31" t="n">
         <v>55</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="31" t="n">
@@ -6433,15 +6571,187 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="32" t="n">
         <v>0.2</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>320</v>
-      </c>
+        <v>327</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="7" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>330</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="18" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="18" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="18" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="18" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="18" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
+        <v>342</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="18" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="18" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="s">
+        <v>346</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="D27" s="8"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="B29" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D29" s="6"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="B30" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="18" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D30" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="B31" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="D31" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6459,7 +6769,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF21"/>
+  <dimension ref="A1:AG21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -6469,7 +6779,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>321</v>
+        <v>354</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -6502,10 +6812,11 @@
       <c r="AD1" s="6"/>
       <c r="AE1" s="6"/>
       <c r="AF1" s="6"/>
+      <c r="AG1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>322</v>
+        <v>355</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -6538,10 +6849,11 @@
       <c r="AD2" s="6"/>
       <c r="AE2" s="6"/>
       <c r="AF2" s="6"/>
+      <c r="AG2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>323</v>
+        <v>356</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -6574,6 +6886,7 @@
       <c r="AD3" s="6"/>
       <c r="AE3" s="6"/>
       <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6"/>
@@ -6608,10 +6921,11 @@
       <c r="AD4" s="6"/>
       <c r="AE4" s="6"/>
       <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>324</v>
+        <v>357</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -6644,40 +6958,41 @@
       <c r="AD5" s="6"/>
       <c r="AE5" s="6"/>
       <c r="AF5" s="6"/>
+      <c r="AG5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>325</v>
+        <v>358</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>327</v>
+        <v>360</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>330</v>
+        <v>363</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>331</v>
+        <v>364</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>332</v>
+        <v>365</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>333</v>
+        <v>366</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>334</v>
+        <v>367</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>335</v>
+        <v>368</v>
       </c>
       <c r="L6" s="8" t="s">
         <v>34</v>
@@ -6742,13 +7057,16 @@
       <c r="AF6" s="8" t="s">
         <v>107</v>
       </c>
+      <c r="AG6" s="8" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>336</v>
+        <v>369</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>337</v>
+        <v>370</v>
       </c>
       <c r="C7" s="33" t="n">
         <v>98048.85</v>
@@ -6840,15 +7158,18 @@
         <v>1</v>
       </c>
       <c r="AF7" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AG7" s="18" t="n">
+        <v>190</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>338</v>
+        <v>371</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>337</v>
+        <v>370</v>
       </c>
       <c r="C8" s="33" t="n">
         <v>91172.79</v>
@@ -6940,7 +7261,10 @@
         <v>3</v>
       </c>
       <c r="AF8" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AG8" s="18" t="n">
+        <v>190</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6976,10 +7300,11 @@
       <c r="AD9" s="6"/>
       <c r="AE9" s="6"/>
       <c r="AF9" s="6"/>
+      <c r="AG9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>339</v>
+        <v>372</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -7012,22 +7337,23 @@
       <c r="AD10" s="6"/>
       <c r="AE10" s="6"/>
       <c r="AF10" s="6"/>
+      <c r="AG10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>340</v>
+        <v>373</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>341</v>
+        <v>374</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>342</v>
+        <v>375</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>343</v>
+        <v>376</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>344</v>
+        <v>377</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -7056,13 +7382,14 @@
       <c r="AD11" s="6"/>
       <c r="AE11" s="6"/>
       <c r="AF11" s="6"/>
+      <c r="AG11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>345</v>
+        <v>378</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>346</v>
+        <v>379</v>
       </c>
       <c r="C12" s="35" t="n">
         <v>870</v>
@@ -7101,13 +7428,14 @@
       <c r="AD12" s="6"/>
       <c r="AE12" s="6"/>
       <c r="AF12" s="6"/>
+      <c r="AG12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>348</v>
+        <v>381</v>
       </c>
       <c r="C13" s="35" t="n">
         <v>1178</v>
@@ -7146,13 +7474,14 @@
       <c r="AD13" s="6"/>
       <c r="AE13" s="6"/>
       <c r="AF13" s="6"/>
+      <c r="AG13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>349</v>
+        <v>382</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>350</v>
+        <v>383</v>
       </c>
       <c r="C14" s="35" t="n">
         <v>33.75</v>
@@ -7191,13 +7520,14 @@
       <c r="AD14" s="6"/>
       <c r="AE14" s="6"/>
       <c r="AF14" s="6"/>
+      <c r="AG14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>345</v>
+        <v>378</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>351</v>
+        <v>384</v>
       </c>
       <c r="C15" s="35" t="n">
         <v>174</v>
@@ -7236,13 +7566,14 @@
       <c r="AD15" s="6"/>
       <c r="AE15" s="6"/>
       <c r="AF15" s="6"/>
+      <c r="AG15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>351</v>
+        <v>384</v>
       </c>
       <c r="C16" s="35" t="n">
         <v>169.34</v>
@@ -7281,13 +7612,14 @@
       <c r="AD16" s="6"/>
       <c r="AE16" s="6"/>
       <c r="AF16" s="6"/>
+      <c r="AG16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>345</v>
+        <v>378</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>352</v>
+        <v>385</v>
       </c>
       <c r="C17" s="35" t="n">
         <v>40</v>
@@ -7326,13 +7658,14 @@
       <c r="AD17" s="6"/>
       <c r="AE17" s="6"/>
       <c r="AF17" s="6"/>
+      <c r="AG17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>353</v>
+        <v>386</v>
       </c>
       <c r="C18" s="35" t="n">
         <v>72</v>
@@ -7371,6 +7704,7 @@
       <c r="AD18" s="6"/>
       <c r="AE18" s="6"/>
       <c r="AF18" s="6"/>
+      <c r="AG18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6"/>
@@ -7405,10 +7739,11 @@
       <c r="AD19" s="6"/>
       <c r="AE19" s="6"/>
       <c r="AF19" s="6"/>
+      <c r="AG19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>354</v>
+        <v>387</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -7441,10 +7776,11 @@
       <c r="AD20" s="6"/>
       <c r="AE20" s="6"/>
       <c r="AF20" s="6"/>
+      <c r="AG20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>355</v>
+        <v>388</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -7477,6 +7813,7 @@
       <c r="AD21" s="6"/>
       <c r="AE21" s="6"/>
       <c r="AF21" s="6"/>
+      <c r="AG21" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>